<commit_message>
Fixing download excel integrity issues
</commit_message>
<xml_diff>
--- a/thaco/color/1_MID_Office.xlsx
+++ b/thaco/color/1_MID_Office.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/gitlocal/thaco/color/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8D9227-D8EE-4849-94DF-BC9D759A0992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8C64F6D-0154-C449-AB4B-3F67CD45938B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38440" yWindow="500" windowWidth="38360" windowHeight="20700" tabRatio="761" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38440" yWindow="500" windowWidth="38360" windowHeight="20700" tabRatio="761" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bảng lương CB-NV" sheetId="1" r:id="rId1"/>
@@ -5850,7 +5850,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="25" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="483">
+  <cellXfs count="479">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -6745,11 +6745,7 @@
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="29" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="55" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="55" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -7015,9 +7011,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="73" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -7062,7 +7055,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="54" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="73" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -7844,88 +7836,88 @@
       <c r="CD2" s="203"/>
     </row>
     <row r="3" spans="1:87" s="2" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="379"/>
-      <c r="B3" s="375"/>
-      <c r="C3" s="375"/>
-      <c r="D3" s="375"/>
-      <c r="E3" s="375"/>
-      <c r="F3" s="375"/>
-      <c r="G3" s="375"/>
-      <c r="H3" s="375"/>
-      <c r="I3" s="375"/>
-      <c r="J3" s="375"/>
-      <c r="K3" s="375"/>
-      <c r="L3" s="375"/>
-      <c r="M3" s="375"/>
-      <c r="N3" s="375"/>
-      <c r="O3" s="375"/>
-      <c r="P3" s="375"/>
-      <c r="Q3" s="375"/>
-      <c r="R3" s="375"/>
-      <c r="S3" s="375"/>
-      <c r="T3" s="375"/>
-      <c r="U3" s="375"/>
-      <c r="V3" s="375"/>
-      <c r="W3" s="375"/>
-      <c r="X3" s="375"/>
-      <c r="Y3" s="375"/>
-      <c r="Z3" s="375"/>
-      <c r="AA3" s="375"/>
-      <c r="AB3" s="375"/>
-      <c r="AC3" s="375"/>
-      <c r="AD3" s="375"/>
-      <c r="AE3" s="375"/>
-      <c r="AF3" s="375"/>
-      <c r="AG3" s="375"/>
-      <c r="AH3" s="375"/>
-      <c r="AI3" s="375"/>
-      <c r="AJ3" s="375"/>
-      <c r="AK3" s="375"/>
-      <c r="AL3" s="375"/>
-      <c r="AM3" s="375"/>
-      <c r="AN3" s="375"/>
-      <c r="AO3" s="375"/>
-      <c r="AP3" s="375"/>
-      <c r="AQ3" s="375"/>
-      <c r="AR3" s="375"/>
-      <c r="AS3" s="375"/>
-      <c r="AT3" s="375"/>
-      <c r="AU3" s="375"/>
-      <c r="AV3" s="375"/>
-      <c r="AW3" s="375"/>
-      <c r="AX3" s="375"/>
-      <c r="AY3" s="375"/>
-      <c r="AZ3" s="375"/>
-      <c r="BA3" s="375"/>
-      <c r="BB3" s="375"/>
-      <c r="BC3" s="375"/>
-      <c r="BD3" s="375"/>
-      <c r="BE3" s="375"/>
-      <c r="BF3" s="375"/>
-      <c r="BG3" s="375"/>
-      <c r="BH3" s="375"/>
-      <c r="BI3" s="375"/>
-      <c r="BJ3" s="375"/>
-      <c r="BK3" s="375"/>
-      <c r="BL3" s="375"/>
-      <c r="BM3" s="375"/>
-      <c r="BN3" s="375"/>
-      <c r="BO3" s="375"/>
-      <c r="BP3" s="375"/>
-      <c r="BQ3" s="375"/>
-      <c r="BR3" s="375"/>
-      <c r="BS3" s="375"/>
-      <c r="BT3" s="375"/>
-      <c r="BU3" s="375"/>
+      <c r="A3" s="377"/>
+      <c r="B3" s="373"/>
+      <c r="C3" s="373"/>
+      <c r="D3" s="373"/>
+      <c r="E3" s="373"/>
+      <c r="F3" s="373"/>
+      <c r="G3" s="373"/>
+      <c r="H3" s="373"/>
+      <c r="I3" s="373"/>
+      <c r="J3" s="373"/>
+      <c r="K3" s="373"/>
+      <c r="L3" s="373"/>
+      <c r="M3" s="373"/>
+      <c r="N3" s="373"/>
+      <c r="O3" s="373"/>
+      <c r="P3" s="373"/>
+      <c r="Q3" s="373"/>
+      <c r="R3" s="373"/>
+      <c r="S3" s="373"/>
+      <c r="T3" s="373"/>
+      <c r="U3" s="373"/>
+      <c r="V3" s="373"/>
+      <c r="W3" s="373"/>
+      <c r="X3" s="373"/>
+      <c r="Y3" s="373"/>
+      <c r="Z3" s="373"/>
+      <c r="AA3" s="373"/>
+      <c r="AB3" s="373"/>
+      <c r="AC3" s="373"/>
+      <c r="AD3" s="373"/>
+      <c r="AE3" s="373"/>
+      <c r="AF3" s="373"/>
+      <c r="AG3" s="373"/>
+      <c r="AH3" s="373"/>
+      <c r="AI3" s="373"/>
+      <c r="AJ3" s="373"/>
+      <c r="AK3" s="373"/>
+      <c r="AL3" s="373"/>
+      <c r="AM3" s="373"/>
+      <c r="AN3" s="373"/>
+      <c r="AO3" s="373"/>
+      <c r="AP3" s="373"/>
+      <c r="AQ3" s="373"/>
+      <c r="AR3" s="373"/>
+      <c r="AS3" s="373"/>
+      <c r="AT3" s="373"/>
+      <c r="AU3" s="373"/>
+      <c r="AV3" s="373"/>
+      <c r="AW3" s="373"/>
+      <c r="AX3" s="373"/>
+      <c r="AY3" s="373"/>
+      <c r="AZ3" s="373"/>
+      <c r="BA3" s="373"/>
+      <c r="BB3" s="373"/>
+      <c r="BC3" s="373"/>
+      <c r="BD3" s="373"/>
+      <c r="BE3" s="373"/>
+      <c r="BF3" s="373"/>
+      <c r="BG3" s="373"/>
+      <c r="BH3" s="373"/>
+      <c r="BI3" s="373"/>
+      <c r="BJ3" s="373"/>
+      <c r="BK3" s="373"/>
+      <c r="BL3" s="373"/>
+      <c r="BM3" s="373"/>
+      <c r="BN3" s="373"/>
+      <c r="BO3" s="373"/>
+      <c r="BP3" s="373"/>
+      <c r="BQ3" s="373"/>
+      <c r="BR3" s="373"/>
+      <c r="BS3" s="373"/>
+      <c r="BT3" s="373"/>
+      <c r="BU3" s="373"/>
       <c r="BV3" s="205"/>
-      <c r="BW3" s="374" t="s">
+      <c r="BW3" s="372" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="375"/>
-      <c r="BY3" s="375"/>
-      <c r="BZ3" s="375"/>
-      <c r="CA3" s="375"/>
-      <c r="CB3" s="375"/>
+      <c r="BX3" s="373"/>
+      <c r="BY3" s="373"/>
+      <c r="BZ3" s="373"/>
+      <c r="CA3" s="373"/>
+      <c r="CB3" s="373"/>
       <c r="CC3" s="207"/>
       <c r="CD3" s="207"/>
     </row>
@@ -8003,12 +7995,12 @@
       <c r="BT4" s="208"/>
       <c r="BU4" s="208"/>
       <c r="BV4" s="208"/>
-      <c r="BW4" s="375"/>
-      <c r="BX4" s="375"/>
-      <c r="BY4" s="375"/>
-      <c r="BZ4" s="375"/>
-      <c r="CA4" s="375"/>
-      <c r="CB4" s="375"/>
+      <c r="BW4" s="373"/>
+      <c r="BX4" s="373"/>
+      <c r="BY4" s="373"/>
+      <c r="BZ4" s="373"/>
+      <c r="CA4" s="373"/>
+      <c r="CB4" s="373"/>
       <c r="CC4" s="207"/>
       <c r="CD4" s="207"/>
     </row>
@@ -8086,12 +8078,12 @@
       <c r="BT5" s="208"/>
       <c r="BU5" s="208"/>
       <c r="BV5" s="208"/>
-      <c r="BW5" s="375"/>
-      <c r="BX5" s="375"/>
-      <c r="BY5" s="375"/>
-      <c r="BZ5" s="375"/>
-      <c r="CA5" s="375"/>
-      <c r="CB5" s="375"/>
+      <c r="BW5" s="373"/>
+      <c r="BX5" s="373"/>
+      <c r="BY5" s="373"/>
+      <c r="BZ5" s="373"/>
+      <c r="CA5" s="373"/>
+      <c r="CB5" s="373"/>
       <c r="CC5" s="207"/>
       <c r="CD5" s="207"/>
     </row>
@@ -8167,12 +8159,12 @@
       <c r="BT6" s="210"/>
       <c r="BU6" s="210"/>
       <c r="BV6" s="210"/>
-      <c r="BW6" s="375"/>
-      <c r="BX6" s="375"/>
-      <c r="BY6" s="375"/>
-      <c r="BZ6" s="375"/>
-      <c r="CA6" s="375"/>
-      <c r="CB6" s="375"/>
+      <c r="BW6" s="373"/>
+      <c r="BX6" s="373"/>
+      <c r="BY6" s="373"/>
+      <c r="BZ6" s="373"/>
+      <c r="CA6" s="373"/>
+      <c r="CB6" s="373"/>
       <c r="CC6" s="207"/>
       <c r="CD6" s="207"/>
     </row>
@@ -8312,356 +8304,356 @@
       </c>
     </row>
     <row r="8" spans="1:87" s="213" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="373" t="s">
+      <c r="A8" s="371" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="381" t="s">
+      <c r="B8" s="379" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="349" t="s">
+      <c r="C8" s="347" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="360" t="s">
+      <c r="D8" s="358" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="360" t="s">
+      <c r="E8" s="358" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="349" t="s">
+      <c r="F8" s="347" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="361" t="s">
+      <c r="G8" s="359" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="362" t="s">
+      <c r="H8" s="360" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="362" t="s">
+      <c r="I8" s="360" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="356" t="s">
+      <c r="J8" s="354" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="372" t="s">
+      <c r="K8" s="370" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="353"/>
-      <c r="M8" s="353"/>
-      <c r="N8" s="353"/>
-      <c r="O8" s="353"/>
-      <c r="P8" s="353"/>
-      <c r="Q8" s="353"/>
-      <c r="R8" s="353"/>
-      <c r="S8" s="353"/>
-      <c r="T8" s="353"/>
-      <c r="U8" s="353"/>
-      <c r="V8" s="353"/>
-      <c r="W8" s="353"/>
-      <c r="X8" s="353"/>
-      <c r="Y8" s="352" t="s">
+      <c r="L8" s="351"/>
+      <c r="M8" s="351"/>
+      <c r="N8" s="351"/>
+      <c r="O8" s="351"/>
+      <c r="P8" s="351"/>
+      <c r="Q8" s="351"/>
+      <c r="R8" s="351"/>
+      <c r="S8" s="351"/>
+      <c r="T8" s="351"/>
+      <c r="U8" s="351"/>
+      <c r="V8" s="351"/>
+      <c r="W8" s="351"/>
+      <c r="X8" s="351"/>
+      <c r="Y8" s="350" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="353"/>
-      <c r="AA8" s="353"/>
-      <c r="AB8" s="353"/>
-      <c r="AC8" s="353"/>
-      <c r="AD8" s="353"/>
-      <c r="AE8" s="353"/>
-      <c r="AF8" s="353"/>
-      <c r="AG8" s="353"/>
-      <c r="AH8" s="353"/>
-      <c r="AI8" s="353"/>
-      <c r="AJ8" s="353"/>
-      <c r="AK8" s="353"/>
-      <c r="AL8" s="353"/>
-      <c r="AM8" s="353"/>
-      <c r="AN8" s="353"/>
-      <c r="AO8" s="354"/>
-      <c r="AP8" s="356" t="s">
+      <c r="Z8" s="351"/>
+      <c r="AA8" s="351"/>
+      <c r="AB8" s="351"/>
+      <c r="AC8" s="351"/>
+      <c r="AD8" s="351"/>
+      <c r="AE8" s="351"/>
+      <c r="AF8" s="351"/>
+      <c r="AG8" s="351"/>
+      <c r="AH8" s="351"/>
+      <c r="AI8" s="351"/>
+      <c r="AJ8" s="351"/>
+      <c r="AK8" s="351"/>
+      <c r="AL8" s="351"/>
+      <c r="AM8" s="351"/>
+      <c r="AN8" s="351"/>
+      <c r="AO8" s="352"/>
+      <c r="AP8" s="354" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="356" t="s">
+      <c r="AQ8" s="354" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="356" t="s">
+      <c r="AR8" s="354" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="356" t="s">
+      <c r="AS8" s="354" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="356" t="s">
+      <c r="AT8" s="354" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="356" t="s">
+      <c r="AU8" s="354" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="349" t="s">
+      <c r="AV8" s="347" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="350" t="s">
+      <c r="AW8" s="348" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="339" t="s">
+      <c r="AX8" s="337" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="358" t="s">
+      <c r="AY8" s="356" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="353"/>
-      <c r="BA8" s="353"/>
-      <c r="BB8" s="353"/>
-      <c r="BC8" s="353"/>
-      <c r="BD8" s="353"/>
-      <c r="BE8" s="353"/>
-      <c r="BF8" s="353"/>
-      <c r="BG8" s="353"/>
-      <c r="BH8" s="353"/>
-      <c r="BI8" s="353"/>
-      <c r="BJ8" s="353"/>
-      <c r="BK8" s="353"/>
-      <c r="BL8" s="353"/>
-      <c r="BM8" s="353"/>
-      <c r="BN8" s="353"/>
-      <c r="BO8" s="353"/>
-      <c r="BP8" s="353"/>
-      <c r="BQ8" s="354"/>
-      <c r="BR8" s="342" t="s">
+      <c r="AZ8" s="351"/>
+      <c r="BA8" s="351"/>
+      <c r="BB8" s="351"/>
+      <c r="BC8" s="351"/>
+      <c r="BD8" s="351"/>
+      <c r="BE8" s="351"/>
+      <c r="BF8" s="351"/>
+      <c r="BG8" s="351"/>
+      <c r="BH8" s="351"/>
+      <c r="BI8" s="351"/>
+      <c r="BJ8" s="351"/>
+      <c r="BK8" s="351"/>
+      <c r="BL8" s="351"/>
+      <c r="BM8" s="351"/>
+      <c r="BN8" s="351"/>
+      <c r="BO8" s="351"/>
+      <c r="BP8" s="351"/>
+      <c r="BQ8" s="352"/>
+      <c r="BR8" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="BS8" s="343"/>
-      <c r="BT8" s="349" t="s">
+      <c r="BS8" s="341"/>
+      <c r="BT8" s="347" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="336" t="s">
+      <c r="BU8" s="334" t="s">
         <v>28</v>
       </c>
       <c r="BV8" s="3"/>
-      <c r="BW8" s="391" t="s">
+      <c r="BW8" s="389" t="s">
         <v>29</v>
       </c>
-      <c r="BX8" s="382" t="s">
+      <c r="BX8" s="380" t="s">
         <v>30</v>
       </c>
-      <c r="BY8" s="383"/>
-      <c r="BZ8" s="383"/>
-      <c r="CA8" s="384"/>
-      <c r="CB8" s="344" t="s">
+      <c r="BY8" s="381"/>
+      <c r="BZ8" s="381"/>
+      <c r="CA8" s="382"/>
+      <c r="CB8" s="342" t="s">
         <v>31</v>
       </c>
-      <c r="CC8" s="376" t="s">
+      <c r="CC8" s="374" t="s">
         <v>32</v>
       </c>
-      <c r="CD8" s="330" t="s">
+      <c r="CD8" s="374" t="s">
         <v>33</v>
       </c>
       <c r="CH8" s="150"/>
       <c r="CI8" s="150"/>
     </row>
     <row r="9" spans="1:87" s="213" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="363"/>
-      <c r="B9" s="334"/>
-      <c r="C9" s="334"/>
-      <c r="D9" s="334"/>
-      <c r="E9" s="334"/>
-      <c r="F9" s="334"/>
-      <c r="G9" s="340"/>
-      <c r="H9" s="363"/>
-      <c r="I9" s="363"/>
-      <c r="J9" s="331"/>
-      <c r="K9" s="366" t="s">
+      <c r="A9" s="361"/>
+      <c r="B9" s="332"/>
+      <c r="C9" s="332"/>
+      <c r="D9" s="332"/>
+      <c r="E9" s="332"/>
+      <c r="F9" s="332"/>
+      <c r="G9" s="338"/>
+      <c r="H9" s="361"/>
+      <c r="I9" s="361"/>
+      <c r="J9" s="330"/>
+      <c r="K9" s="364" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="366" t="s">
+      <c r="L9" s="364" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="366" t="s">
+      <c r="M9" s="364" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="366" t="s">
+      <c r="N9" s="364" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="366" t="s">
+      <c r="O9" s="364" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="366" t="s">
+      <c r="P9" s="364" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="366" t="s">
+      <c r="Q9" s="364" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="366" t="s">
+      <c r="R9" s="364" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="366" t="s">
+      <c r="S9" s="364" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="366" t="s">
+      <c r="T9" s="364" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="366" t="s">
+      <c r="U9" s="364" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="367" t="s">
+      <c r="V9" s="365" t="s">
         <v>45</v>
       </c>
-      <c r="W9" s="343"/>
-      <c r="X9" s="366" t="s">
+      <c r="W9" s="341"/>
+      <c r="X9" s="364" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="333" t="s">
+      <c r="Y9" s="331" t="s">
         <v>154</v>
       </c>
-      <c r="Z9" s="333" t="s">
+      <c r="Z9" s="331" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="333" t="s">
+      <c r="AA9" s="331" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="333" t="s">
+      <c r="AB9" s="331" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="333" t="s">
+      <c r="AC9" s="331" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="333" t="s">
+      <c r="AD9" s="331" t="s">
         <v>52</v>
       </c>
-      <c r="AE9" s="333" t="s">
+      <c r="AE9" s="331" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="333" t="s">
+      <c r="AF9" s="331" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="333" t="s">
+      <c r="AG9" s="331" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="333" t="s">
+      <c r="AH9" s="331" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="333" t="s">
+      <c r="AI9" s="331" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="357" t="s">
+      <c r="AJ9" s="355" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="336" t="s">
+      <c r="AK9" s="334" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="339" t="s">
+      <c r="AL9" s="337" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="333" t="s">
+      <c r="AM9" s="331" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="349" t="s">
+      <c r="AN9" s="347" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="349" t="s">
+      <c r="AO9" s="347" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="331"/>
-      <c r="AQ9" s="331"/>
-      <c r="AR9" s="331"/>
-      <c r="AS9" s="331"/>
-      <c r="AT9" s="331"/>
-      <c r="AU9" s="331"/>
-      <c r="AV9" s="334"/>
-      <c r="AW9" s="331"/>
-      <c r="AX9" s="340"/>
-      <c r="AY9" s="346" t="s">
+      <c r="AP9" s="330"/>
+      <c r="AQ9" s="330"/>
+      <c r="AR9" s="330"/>
+      <c r="AS9" s="330"/>
+      <c r="AT9" s="330"/>
+      <c r="AU9" s="330"/>
+      <c r="AV9" s="332"/>
+      <c r="AW9" s="330"/>
+      <c r="AX9" s="338"/>
+      <c r="AY9" s="344" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="347"/>
-      <c r="BA9" s="347"/>
-      <c r="BB9" s="347"/>
-      <c r="BC9" s="347"/>
-      <c r="BD9" s="347"/>
-      <c r="BE9" s="347"/>
-      <c r="BF9" s="347"/>
-      <c r="BG9" s="347"/>
-      <c r="BH9" s="347"/>
-      <c r="BI9" s="347"/>
-      <c r="BJ9" s="347"/>
-      <c r="BK9" s="347"/>
-      <c r="BL9" s="348"/>
-      <c r="BM9" s="346" t="s">
+      <c r="AZ9" s="345"/>
+      <c r="BA9" s="345"/>
+      <c r="BB9" s="345"/>
+      <c r="BC9" s="345"/>
+      <c r="BD9" s="345"/>
+      <c r="BE9" s="345"/>
+      <c r="BF9" s="345"/>
+      <c r="BG9" s="345"/>
+      <c r="BH9" s="345"/>
+      <c r="BI9" s="345"/>
+      <c r="BJ9" s="345"/>
+      <c r="BK9" s="345"/>
+      <c r="BL9" s="346"/>
+      <c r="BM9" s="344" t="s">
         <v>64</v>
       </c>
-      <c r="BN9" s="347"/>
-      <c r="BO9" s="347"/>
-      <c r="BP9" s="347"/>
-      <c r="BQ9" s="348"/>
-      <c r="BR9" s="365" t="s">
+      <c r="BN9" s="345"/>
+      <c r="BO9" s="345"/>
+      <c r="BP9" s="345"/>
+      <c r="BQ9" s="346"/>
+      <c r="BR9" s="363" t="s">
         <v>65</v>
       </c>
-      <c r="BS9" s="365" t="s">
+      <c r="BS9" s="363" t="s">
         <v>66</v>
       </c>
-      <c r="BT9" s="334"/>
-      <c r="BU9" s="337"/>
+      <c r="BT9" s="332"/>
+      <c r="BU9" s="335"/>
       <c r="BV9" s="3"/>
-      <c r="BW9" s="392"/>
-      <c r="BX9" s="385"/>
-      <c r="BY9" s="386"/>
-      <c r="BZ9" s="386"/>
-      <c r="CA9" s="387"/>
-      <c r="CB9" s="334"/>
-      <c r="CC9" s="377"/>
-      <c r="CD9" s="331"/>
+      <c r="BW9" s="390"/>
+      <c r="BX9" s="383"/>
+      <c r="BY9" s="384"/>
+      <c r="BZ9" s="384"/>
+      <c r="CA9" s="385"/>
+      <c r="CB9" s="332"/>
+      <c r="CC9" s="375"/>
+      <c r="CD9" s="375"/>
       <c r="CH9" s="150"/>
       <c r="CI9" s="150"/>
     </row>
     <row r="10" spans="1:87" s="214" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="363"/>
-      <c r="B10" s="334"/>
-      <c r="C10" s="334"/>
-      <c r="D10" s="334"/>
-      <c r="E10" s="334"/>
-      <c r="F10" s="334"/>
-      <c r="G10" s="340"/>
-      <c r="H10" s="363"/>
-      <c r="I10" s="363"/>
-      <c r="J10" s="331"/>
-      <c r="K10" s="363"/>
-      <c r="L10" s="363"/>
-      <c r="M10" s="363"/>
-      <c r="N10" s="363"/>
-      <c r="O10" s="363"/>
-      <c r="P10" s="363"/>
-      <c r="Q10" s="363"/>
-      <c r="R10" s="363"/>
-      <c r="S10" s="363"/>
-      <c r="T10" s="363"/>
-      <c r="U10" s="363"/>
-      <c r="V10" s="368"/>
-      <c r="W10" s="369"/>
-      <c r="X10" s="363"/>
-      <c r="Y10" s="334"/>
-      <c r="Z10" s="334"/>
-      <c r="AA10" s="334"/>
-      <c r="AB10" s="334"/>
-      <c r="AC10" s="334"/>
-      <c r="AD10" s="334"/>
-      <c r="AE10" s="334"/>
-      <c r="AF10" s="334"/>
-      <c r="AG10" s="334"/>
-      <c r="AH10" s="334"/>
-      <c r="AI10" s="334"/>
-      <c r="AJ10" s="340"/>
-      <c r="AK10" s="337"/>
-      <c r="AL10" s="340"/>
-      <c r="AM10" s="334"/>
-      <c r="AN10" s="334"/>
-      <c r="AO10" s="334"/>
-      <c r="AP10" s="331"/>
-      <c r="AQ10" s="331"/>
-      <c r="AR10" s="331"/>
-      <c r="AS10" s="331"/>
-      <c r="AT10" s="331"/>
-      <c r="AU10" s="331"/>
-      <c r="AV10" s="334"/>
-      <c r="AW10" s="331"/>
-      <c r="AX10" s="340"/>
+      <c r="A10" s="361"/>
+      <c r="B10" s="332"/>
+      <c r="C10" s="332"/>
+      <c r="D10" s="332"/>
+      <c r="E10" s="332"/>
+      <c r="F10" s="332"/>
+      <c r="G10" s="338"/>
+      <c r="H10" s="361"/>
+      <c r="I10" s="361"/>
+      <c r="J10" s="330"/>
+      <c r="K10" s="361"/>
+      <c r="L10" s="361"/>
+      <c r="M10" s="361"/>
+      <c r="N10" s="361"/>
+      <c r="O10" s="361"/>
+      <c r="P10" s="361"/>
+      <c r="Q10" s="361"/>
+      <c r="R10" s="361"/>
+      <c r="S10" s="361"/>
+      <c r="T10" s="361"/>
+      <c r="U10" s="361"/>
+      <c r="V10" s="366"/>
+      <c r="W10" s="367"/>
+      <c r="X10" s="361"/>
+      <c r="Y10" s="332"/>
+      <c r="Z10" s="332"/>
+      <c r="AA10" s="332"/>
+      <c r="AB10" s="332"/>
+      <c r="AC10" s="332"/>
+      <c r="AD10" s="332"/>
+      <c r="AE10" s="332"/>
+      <c r="AF10" s="332"/>
+      <c r="AG10" s="332"/>
+      <c r="AH10" s="332"/>
+      <c r="AI10" s="332"/>
+      <c r="AJ10" s="338"/>
+      <c r="AK10" s="335"/>
+      <c r="AL10" s="338"/>
+      <c r="AM10" s="332"/>
+      <c r="AN10" s="332"/>
+      <c r="AO10" s="332"/>
+      <c r="AP10" s="330"/>
+      <c r="AQ10" s="330"/>
+      <c r="AR10" s="330"/>
+      <c r="AS10" s="330"/>
+      <c r="AT10" s="330"/>
+      <c r="AU10" s="330"/>
+      <c r="AV10" s="332"/>
+      <c r="AW10" s="330"/>
+      <c r="AX10" s="338"/>
       <c r="AY10" s="29" t="s">
         <v>67</v>
       </c>
@@ -8671,67 +8663,67 @@
       <c r="BA10" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="BB10" s="380" t="s">
+      <c r="BB10" s="378" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="359" t="s">
+      <c r="BC10" s="357" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="359" t="s">
+      <c r="BD10" s="357" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="355" t="s">
+      <c r="BE10" s="353" t="s">
         <v>73</v>
       </c>
-      <c r="BF10" s="355" t="s">
+      <c r="BF10" s="353" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="394" t="s">
+      <c r="BG10" s="392" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="359" t="s">
+      <c r="BH10" s="357" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="370" t="s">
+      <c r="BI10" s="368" t="s">
         <v>77</v>
       </c>
-      <c r="BJ10" s="355" t="s">
+      <c r="BJ10" s="353" t="s">
         <v>78</v>
       </c>
-      <c r="BK10" s="355" t="s">
+      <c r="BK10" s="353" t="s">
         <v>79</v>
       </c>
-      <c r="BL10" s="349" t="s">
+      <c r="BL10" s="347" t="s">
         <v>80</v>
       </c>
-      <c r="BM10" s="359" t="s">
+      <c r="BM10" s="357" t="s">
         <v>81</v>
       </c>
-      <c r="BN10" s="350" t="s">
+      <c r="BN10" s="348" t="s">
         <v>82</v>
       </c>
-      <c r="BO10" s="359" t="s">
+      <c r="BO10" s="357" t="s">
         <v>83</v>
       </c>
-      <c r="BP10" s="350" t="s">
+      <c r="BP10" s="348" t="s">
         <v>84</v>
       </c>
-      <c r="BQ10" s="350" t="s">
+      <c r="BQ10" s="348" t="s">
         <v>85</v>
       </c>
-      <c r="BR10" s="363"/>
-      <c r="BS10" s="363"/>
-      <c r="BT10" s="334"/>
-      <c r="BU10" s="337"/>
+      <c r="BR10" s="361"/>
+      <c r="BS10" s="361"/>
+      <c r="BT10" s="332"/>
+      <c r="BU10" s="335"/>
       <c r="BV10" s="3"/>
-      <c r="BW10" s="392"/>
-      <c r="BX10" s="388"/>
-      <c r="BY10" s="389"/>
-      <c r="BZ10" s="389"/>
-      <c r="CA10" s="390"/>
-      <c r="CB10" s="334"/>
-      <c r="CC10" s="377"/>
-      <c r="CD10" s="331"/>
+      <c r="BW10" s="390"/>
+      <c r="BX10" s="386"/>
+      <c r="BY10" s="387"/>
+      <c r="BZ10" s="387"/>
+      <c r="CA10" s="388"/>
+      <c r="CB10" s="332"/>
+      <c r="CC10" s="375"/>
+      <c r="CD10" s="375"/>
       <c r="CE10" s="228" t="s">
         <v>3</v>
       </c>
@@ -8739,60 +8731,60 @@
       <c r="CI10" s="150"/>
     </row>
     <row r="11" spans="1:87" s="214" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="364"/>
-      <c r="B11" s="335"/>
-      <c r="C11" s="335"/>
-      <c r="D11" s="335"/>
-      <c r="E11" s="335"/>
-      <c r="F11" s="335"/>
-      <c r="G11" s="341"/>
-      <c r="H11" s="364"/>
-      <c r="I11" s="364"/>
-      <c r="J11" s="351"/>
-      <c r="K11" s="364"/>
-      <c r="L11" s="364"/>
-      <c r="M11" s="364"/>
-      <c r="N11" s="364"/>
-      <c r="O11" s="364"/>
-      <c r="P11" s="364"/>
-      <c r="Q11" s="364"/>
-      <c r="R11" s="364"/>
-      <c r="S11" s="364"/>
-      <c r="T11" s="364"/>
-      <c r="U11" s="364"/>
+      <c r="A11" s="362"/>
+      <c r="B11" s="333"/>
+      <c r="C11" s="333"/>
+      <c r="D11" s="333"/>
+      <c r="E11" s="333"/>
+      <c r="F11" s="333"/>
+      <c r="G11" s="339"/>
+      <c r="H11" s="362"/>
+      <c r="I11" s="362"/>
+      <c r="J11" s="349"/>
+      <c r="K11" s="362"/>
+      <c r="L11" s="362"/>
+      <c r="M11" s="362"/>
+      <c r="N11" s="362"/>
+      <c r="O11" s="362"/>
+      <c r="P11" s="362"/>
+      <c r="Q11" s="362"/>
+      <c r="R11" s="362"/>
+      <c r="S11" s="362"/>
+      <c r="T11" s="362"/>
+      <c r="U11" s="362"/>
       <c r="V11" s="178" t="s">
         <v>86</v>
       </c>
       <c r="W11" s="178" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="364"/>
-      <c r="Y11" s="335"/>
-      <c r="Z11" s="335"/>
-      <c r="AA11" s="335"/>
-      <c r="AB11" s="335"/>
-      <c r="AC11" s="335"/>
-      <c r="AD11" s="335"/>
-      <c r="AE11" s="335"/>
-      <c r="AF11" s="335"/>
-      <c r="AG11" s="335"/>
-      <c r="AH11" s="335"/>
-      <c r="AI11" s="335"/>
-      <c r="AJ11" s="341"/>
-      <c r="AK11" s="338"/>
-      <c r="AL11" s="341"/>
-      <c r="AM11" s="335"/>
-      <c r="AN11" s="335"/>
-      <c r="AO11" s="335"/>
-      <c r="AP11" s="351"/>
-      <c r="AQ11" s="351"/>
-      <c r="AR11" s="351"/>
-      <c r="AS11" s="351"/>
-      <c r="AT11" s="351"/>
-      <c r="AU11" s="351"/>
-      <c r="AV11" s="335"/>
-      <c r="AW11" s="351"/>
-      <c r="AX11" s="341"/>
+      <c r="X11" s="362"/>
+      <c r="Y11" s="333"/>
+      <c r="Z11" s="333"/>
+      <c r="AA11" s="333"/>
+      <c r="AB11" s="333"/>
+      <c r="AC11" s="333"/>
+      <c r="AD11" s="333"/>
+      <c r="AE11" s="333"/>
+      <c r="AF11" s="333"/>
+      <c r="AG11" s="333"/>
+      <c r="AH11" s="333"/>
+      <c r="AI11" s="333"/>
+      <c r="AJ11" s="339"/>
+      <c r="AK11" s="336"/>
+      <c r="AL11" s="339"/>
+      <c r="AM11" s="333"/>
+      <c r="AN11" s="333"/>
+      <c r="AO11" s="333"/>
+      <c r="AP11" s="349"/>
+      <c r="AQ11" s="349"/>
+      <c r="AR11" s="349"/>
+      <c r="AS11" s="349"/>
+      <c r="AT11" s="349"/>
+      <c r="AU11" s="349"/>
+      <c r="AV11" s="333"/>
+      <c r="AW11" s="349"/>
+      <c r="AX11" s="339"/>
       <c r="AY11" s="229" t="s">
         <v>88</v>
       </c>
@@ -8802,28 +8794,28 @@
       <c r="BA11" s="229" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="335"/>
-      <c r="BC11" s="351"/>
-      <c r="BD11" s="351"/>
-      <c r="BE11" s="335"/>
-      <c r="BF11" s="335"/>
-      <c r="BG11" s="364"/>
-      <c r="BH11" s="351"/>
-      <c r="BI11" s="371"/>
-      <c r="BJ11" s="335"/>
-      <c r="BK11" s="335"/>
-      <c r="BL11" s="335"/>
-      <c r="BM11" s="351"/>
-      <c r="BN11" s="351"/>
-      <c r="BO11" s="351"/>
-      <c r="BP11" s="351"/>
-      <c r="BQ11" s="351"/>
-      <c r="BR11" s="364"/>
-      <c r="BS11" s="364"/>
-      <c r="BT11" s="335"/>
-      <c r="BU11" s="338"/>
+      <c r="BB11" s="333"/>
+      <c r="BC11" s="349"/>
+      <c r="BD11" s="349"/>
+      <c r="BE11" s="333"/>
+      <c r="BF11" s="333"/>
+      <c r="BG11" s="362"/>
+      <c r="BH11" s="349"/>
+      <c r="BI11" s="369"/>
+      <c r="BJ11" s="333"/>
+      <c r="BK11" s="333"/>
+      <c r="BL11" s="333"/>
+      <c r="BM11" s="349"/>
+      <c r="BN11" s="349"/>
+      <c r="BO11" s="349"/>
+      <c r="BP11" s="349"/>
+      <c r="BQ11" s="349"/>
+      <c r="BR11" s="362"/>
+      <c r="BS11" s="362"/>
+      <c r="BT11" s="333"/>
+      <c r="BU11" s="336"/>
       <c r="BV11" s="3"/>
-      <c r="BW11" s="393"/>
+      <c r="BW11" s="391"/>
       <c r="BX11" s="237" t="s">
         <v>91</v>
       </c>
@@ -8836,9 +8828,9 @@
       <c r="CA11" s="238" t="s">
         <v>94</v>
       </c>
-      <c r="CB11" s="345"/>
-      <c r="CC11" s="378"/>
-      <c r="CD11" s="332"/>
+      <c r="CB11" s="343"/>
+      <c r="CC11" s="376"/>
+      <c r="CD11" s="376"/>
       <c r="CE11" s="227">
         <v>26</v>
       </c>
@@ -11602,87 +11594,87 @@
       <c r="CD2" s="41"/>
     </row>
     <row r="3" spans="1:87" s="43" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="424"/>
-      <c r="B3" s="415"/>
-      <c r="C3" s="415"/>
-      <c r="D3" s="415"/>
-      <c r="E3" s="415"/>
-      <c r="F3" s="415"/>
-      <c r="G3" s="415"/>
-      <c r="H3" s="415"/>
-      <c r="I3" s="415"/>
-      <c r="J3" s="415"/>
-      <c r="K3" s="415"/>
-      <c r="L3" s="415"/>
-      <c r="M3" s="415"/>
-      <c r="N3" s="415"/>
-      <c r="O3" s="415"/>
-      <c r="P3" s="415"/>
-      <c r="Q3" s="415"/>
-      <c r="R3" s="415"/>
-      <c r="S3" s="415"/>
-      <c r="T3" s="415"/>
-      <c r="U3" s="415"/>
-      <c r="V3" s="415"/>
-      <c r="W3" s="415"/>
-      <c r="X3" s="415"/>
-      <c r="Y3" s="415"/>
-      <c r="Z3" s="415"/>
-      <c r="AA3" s="415"/>
-      <c r="AB3" s="415"/>
-      <c r="AC3" s="415"/>
-      <c r="AD3" s="415"/>
-      <c r="AE3" s="415"/>
-      <c r="AF3" s="415"/>
-      <c r="AG3" s="415"/>
-      <c r="AH3" s="415"/>
-      <c r="AI3" s="415"/>
-      <c r="AJ3" s="415"/>
-      <c r="AK3" s="415"/>
-      <c r="AL3" s="415"/>
-      <c r="AM3" s="415"/>
-      <c r="AN3" s="415"/>
-      <c r="AO3" s="415"/>
-      <c r="AP3" s="415"/>
-      <c r="AQ3" s="415"/>
-      <c r="AR3" s="415"/>
-      <c r="AS3" s="415"/>
-      <c r="AT3" s="415"/>
-      <c r="AU3" s="415"/>
-      <c r="AV3" s="415"/>
-      <c r="AW3" s="415"/>
-      <c r="AX3" s="415"/>
-      <c r="AY3" s="415"/>
-      <c r="AZ3" s="415"/>
-      <c r="BA3" s="415"/>
-      <c r="BB3" s="415"/>
-      <c r="BC3" s="415"/>
-      <c r="BD3" s="415"/>
-      <c r="BE3" s="415"/>
-      <c r="BF3" s="415"/>
-      <c r="BG3" s="415"/>
-      <c r="BH3" s="415"/>
-      <c r="BI3" s="415"/>
-      <c r="BJ3" s="415"/>
-      <c r="BK3" s="415"/>
-      <c r="BL3" s="415"/>
-      <c r="BM3" s="415"/>
-      <c r="BN3" s="415"/>
-      <c r="BO3" s="415"/>
-      <c r="BP3" s="415"/>
-      <c r="BQ3" s="415"/>
-      <c r="BR3" s="415"/>
-      <c r="BS3" s="415"/>
-      <c r="BT3" s="415"/>
-      <c r="BU3" s="415"/>
-      <c r="BW3" s="414" t="s">
+      <c r="A3" s="422"/>
+      <c r="B3" s="413"/>
+      <c r="C3" s="413"/>
+      <c r="D3" s="413"/>
+      <c r="E3" s="413"/>
+      <c r="F3" s="413"/>
+      <c r="G3" s="413"/>
+      <c r="H3" s="413"/>
+      <c r="I3" s="413"/>
+      <c r="J3" s="413"/>
+      <c r="K3" s="413"/>
+      <c r="L3" s="413"/>
+      <c r="M3" s="413"/>
+      <c r="N3" s="413"/>
+      <c r="O3" s="413"/>
+      <c r="P3" s="413"/>
+      <c r="Q3" s="413"/>
+      <c r="R3" s="413"/>
+      <c r="S3" s="413"/>
+      <c r="T3" s="413"/>
+      <c r="U3" s="413"/>
+      <c r="V3" s="413"/>
+      <c r="W3" s="413"/>
+      <c r="X3" s="413"/>
+      <c r="Y3" s="413"/>
+      <c r="Z3" s="413"/>
+      <c r="AA3" s="413"/>
+      <c r="AB3" s="413"/>
+      <c r="AC3" s="413"/>
+      <c r="AD3" s="413"/>
+      <c r="AE3" s="413"/>
+      <c r="AF3" s="413"/>
+      <c r="AG3" s="413"/>
+      <c r="AH3" s="413"/>
+      <c r="AI3" s="413"/>
+      <c r="AJ3" s="413"/>
+      <c r="AK3" s="413"/>
+      <c r="AL3" s="413"/>
+      <c r="AM3" s="413"/>
+      <c r="AN3" s="413"/>
+      <c r="AO3" s="413"/>
+      <c r="AP3" s="413"/>
+      <c r="AQ3" s="413"/>
+      <c r="AR3" s="413"/>
+      <c r="AS3" s="413"/>
+      <c r="AT3" s="413"/>
+      <c r="AU3" s="413"/>
+      <c r="AV3" s="413"/>
+      <c r="AW3" s="413"/>
+      <c r="AX3" s="413"/>
+      <c r="AY3" s="413"/>
+      <c r="AZ3" s="413"/>
+      <c r="BA3" s="413"/>
+      <c r="BB3" s="413"/>
+      <c r="BC3" s="413"/>
+      <c r="BD3" s="413"/>
+      <c r="BE3" s="413"/>
+      <c r="BF3" s="413"/>
+      <c r="BG3" s="413"/>
+      <c r="BH3" s="413"/>
+      <c r="BI3" s="413"/>
+      <c r="BJ3" s="413"/>
+      <c r="BK3" s="413"/>
+      <c r="BL3" s="413"/>
+      <c r="BM3" s="413"/>
+      <c r="BN3" s="413"/>
+      <c r="BO3" s="413"/>
+      <c r="BP3" s="413"/>
+      <c r="BQ3" s="413"/>
+      <c r="BR3" s="413"/>
+      <c r="BS3" s="413"/>
+      <c r="BT3" s="413"/>
+      <c r="BU3" s="413"/>
+      <c r="BW3" s="412" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="415"/>
-      <c r="BY3" s="415"/>
-      <c r="BZ3" s="415"/>
-      <c r="CA3" s="415"/>
-      <c r="CB3" s="415"/>
+      <c r="BX3" s="413"/>
+      <c r="BY3" s="413"/>
+      <c r="BZ3" s="413"/>
+      <c r="CA3" s="413"/>
+      <c r="CB3" s="413"/>
       <c r="CC3" s="42"/>
       <c r="CD3" s="42"/>
       <c r="CE3" s="43" t="s">
@@ -11765,364 +11757,364 @@
       <c r="BS4" s="44"/>
       <c r="BT4" s="44"/>
       <c r="BU4" s="44"/>
-      <c r="BW4" s="415"/>
-      <c r="BX4" s="415"/>
-      <c r="BY4" s="415"/>
-      <c r="BZ4" s="415"/>
-      <c r="CA4" s="415"/>
-      <c r="CB4" s="415"/>
+      <c r="BW4" s="413"/>
+      <c r="BX4" s="413"/>
+      <c r="BY4" s="413"/>
+      <c r="BZ4" s="413"/>
+      <c r="CA4" s="413"/>
+      <c r="CB4" s="413"/>
       <c r="CC4" s="42"/>
       <c r="CD4" s="42"/>
     </row>
     <row r="5" spans="1:87" s="45" customFormat="1">
-      <c r="A5" s="427" t="s">
+      <c r="A5" s="425" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="426" t="s">
+      <c r="B5" s="424" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="400" t="s">
+      <c r="C5" s="398" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="425" t="s">
+      <c r="D5" s="423" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="425" t="s">
+      <c r="E5" s="423" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="400" t="s">
+      <c r="F5" s="398" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="400" t="s">
+      <c r="G5" s="398" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="349" t="s">
+      <c r="H5" s="347" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="349" t="s">
+      <c r="I5" s="347" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="400" t="s">
+      <c r="J5" s="398" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="429" t="s">
+      <c r="K5" s="427" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="411"/>
-      <c r="M5" s="411"/>
-      <c r="N5" s="411"/>
-      <c r="O5" s="411"/>
-      <c r="P5" s="411"/>
-      <c r="Q5" s="411"/>
-      <c r="R5" s="411"/>
-      <c r="S5" s="411"/>
-      <c r="T5" s="411"/>
-      <c r="U5" s="411"/>
-      <c r="V5" s="411"/>
-      <c r="W5" s="411"/>
-      <c r="X5" s="411"/>
-      <c r="Y5" s="400" t="s">
+      <c r="L5" s="409"/>
+      <c r="M5" s="409"/>
+      <c r="N5" s="409"/>
+      <c r="O5" s="409"/>
+      <c r="P5" s="409"/>
+      <c r="Q5" s="409"/>
+      <c r="R5" s="409"/>
+      <c r="S5" s="409"/>
+      <c r="T5" s="409"/>
+      <c r="U5" s="409"/>
+      <c r="V5" s="409"/>
+      <c r="W5" s="409"/>
+      <c r="X5" s="409"/>
+      <c r="Y5" s="398" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="411"/>
-      <c r="AA5" s="411"/>
-      <c r="AB5" s="411"/>
-      <c r="AC5" s="411"/>
-      <c r="AD5" s="411"/>
-      <c r="AE5" s="411"/>
-      <c r="AF5" s="411"/>
-      <c r="AG5" s="411"/>
-      <c r="AH5" s="411"/>
-      <c r="AI5" s="411"/>
-      <c r="AJ5" s="411"/>
-      <c r="AK5" s="411"/>
-      <c r="AL5" s="411"/>
-      <c r="AM5" s="411"/>
-      <c r="AN5" s="411"/>
-      <c r="AO5" s="412"/>
-      <c r="AP5" s="400" t="s">
+      <c r="Z5" s="409"/>
+      <c r="AA5" s="409"/>
+      <c r="AB5" s="409"/>
+      <c r="AC5" s="409"/>
+      <c r="AD5" s="409"/>
+      <c r="AE5" s="409"/>
+      <c r="AF5" s="409"/>
+      <c r="AG5" s="409"/>
+      <c r="AH5" s="409"/>
+      <c r="AI5" s="409"/>
+      <c r="AJ5" s="409"/>
+      <c r="AK5" s="409"/>
+      <c r="AL5" s="409"/>
+      <c r="AM5" s="409"/>
+      <c r="AN5" s="409"/>
+      <c r="AO5" s="410"/>
+      <c r="AP5" s="398" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="400" t="s">
+      <c r="AQ5" s="398" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="400" t="s">
+      <c r="AR5" s="398" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="400" t="s">
+      <c r="AS5" s="398" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="400" t="s">
+      <c r="AT5" s="398" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="400" t="s">
+      <c r="AU5" s="398" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="400" t="s">
+      <c r="AV5" s="398" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="400" t="s">
+      <c r="AW5" s="398" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="400" t="s">
+      <c r="AX5" s="398" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="410" t="s">
+      <c r="AY5" s="408" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="411"/>
-      <c r="BA5" s="411"/>
-      <c r="BB5" s="411"/>
-      <c r="BC5" s="411"/>
-      <c r="BD5" s="411"/>
-      <c r="BE5" s="411"/>
-      <c r="BF5" s="411"/>
-      <c r="BG5" s="411"/>
-      <c r="BH5" s="411"/>
-      <c r="BI5" s="411"/>
-      <c r="BJ5" s="411"/>
-      <c r="BK5" s="411"/>
-      <c r="BL5" s="411"/>
-      <c r="BM5" s="411"/>
-      <c r="BN5" s="411"/>
-      <c r="BO5" s="411"/>
-      <c r="BP5" s="411"/>
-      <c r="BQ5" s="412"/>
-      <c r="BR5" s="416" t="s">
+      <c r="AZ5" s="409"/>
+      <c r="BA5" s="409"/>
+      <c r="BB5" s="409"/>
+      <c r="BC5" s="409"/>
+      <c r="BD5" s="409"/>
+      <c r="BE5" s="409"/>
+      <c r="BF5" s="409"/>
+      <c r="BG5" s="409"/>
+      <c r="BH5" s="409"/>
+      <c r="BI5" s="409"/>
+      <c r="BJ5" s="409"/>
+      <c r="BK5" s="409"/>
+      <c r="BL5" s="409"/>
+      <c r="BM5" s="409"/>
+      <c r="BN5" s="409"/>
+      <c r="BO5" s="409"/>
+      <c r="BP5" s="409"/>
+      <c r="BQ5" s="410"/>
+      <c r="BR5" s="414" t="s">
         <v>26</v>
       </c>
-      <c r="BS5" s="417"/>
-      <c r="BT5" s="410" t="s">
+      <c r="BS5" s="415"/>
+      <c r="BT5" s="408" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="404" t="s">
+      <c r="BU5" s="402" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="407" t="s">
+      <c r="BW5" s="405" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="418" t="s">
+      <c r="BX5" s="416" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="419"/>
-      <c r="BZ5" s="419"/>
-      <c r="CA5" s="417"/>
-      <c r="CB5" s="413" t="s">
+      <c r="BY5" s="417"/>
+      <c r="BZ5" s="417"/>
+      <c r="CA5" s="415"/>
+      <c r="CB5" s="411" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="395" t="s">
+      <c r="CC5" s="393" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="395" t="s">
+      <c r="CD5" s="393" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="46"/>
       <c r="CI5" s="47"/>
     </row>
     <row r="6" spans="1:87" s="45" customFormat="1">
-      <c r="A6" s="396"/>
-      <c r="B6" s="396"/>
-      <c r="C6" s="396"/>
-      <c r="D6" s="396"/>
-      <c r="E6" s="396"/>
-      <c r="F6" s="396"/>
-      <c r="G6" s="396"/>
-      <c r="H6" s="396"/>
-      <c r="I6" s="396"/>
-      <c r="J6" s="396"/>
-      <c r="K6" s="401" t="s">
+      <c r="A6" s="394"/>
+      <c r="B6" s="394"/>
+      <c r="C6" s="394"/>
+      <c r="D6" s="394"/>
+      <c r="E6" s="394"/>
+      <c r="F6" s="394"/>
+      <c r="G6" s="394"/>
+      <c r="H6" s="394"/>
+      <c r="I6" s="394"/>
+      <c r="J6" s="394"/>
+      <c r="K6" s="399" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="401" t="s">
+      <c r="L6" s="399" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="401" t="s">
+      <c r="M6" s="399" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="401" t="s">
+      <c r="N6" s="399" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="401" t="s">
+      <c r="O6" s="399" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="401" t="s">
+      <c r="P6" s="399" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="401" t="s">
+      <c r="Q6" s="399" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="401" t="s">
+      <c r="R6" s="399" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="401" t="s">
+      <c r="S6" s="399" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="401" t="s">
+      <c r="T6" s="399" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="401" t="s">
+      <c r="U6" s="399" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="431" t="s">
+      <c r="V6" s="429" t="s">
         <v>45</v>
       </c>
-      <c r="W6" s="417"/>
-      <c r="X6" s="401" t="s">
+      <c r="W6" s="415"/>
+      <c r="X6" s="399" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="400" t="s">
+      <c r="Y6" s="398" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="400" t="s">
+      <c r="Z6" s="398" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="400" t="s">
+      <c r="AA6" s="398" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="400" t="s">
+      <c r="AB6" s="398" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="349" t="s">
+      <c r="AC6" s="347" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="349" t="s">
+      <c r="AD6" s="347" t="s">
         <v>52</v>
       </c>
-      <c r="AE6" s="349" t="s">
+      <c r="AE6" s="347" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="349" t="s">
+      <c r="AF6" s="347" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="400" t="s">
+      <c r="AG6" s="398" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="349" t="s">
+      <c r="AH6" s="347" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="349" t="s">
+      <c r="AI6" s="347" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="400" t="s">
+      <c r="AJ6" s="398" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="428" t="s">
+      <c r="AK6" s="426" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="400" t="s">
+      <c r="AL6" s="398" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="400" t="s">
+      <c r="AM6" s="398" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="430" t="s">
+      <c r="AN6" s="428" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="400" t="s">
+      <c r="AO6" s="398" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="396"/>
-      <c r="AQ6" s="396"/>
-      <c r="AR6" s="396"/>
-      <c r="AS6" s="396"/>
-      <c r="AT6" s="396"/>
-      <c r="AU6" s="396"/>
-      <c r="AV6" s="396"/>
-      <c r="AW6" s="396"/>
-      <c r="AX6" s="396"/>
-      <c r="AY6" s="410" t="s">
+      <c r="AP6" s="394"/>
+      <c r="AQ6" s="394"/>
+      <c r="AR6" s="394"/>
+      <c r="AS6" s="394"/>
+      <c r="AT6" s="394"/>
+      <c r="AU6" s="394"/>
+      <c r="AV6" s="394"/>
+      <c r="AW6" s="394"/>
+      <c r="AX6" s="394"/>
+      <c r="AY6" s="408" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="411"/>
-      <c r="BA6" s="411"/>
-      <c r="BB6" s="411"/>
-      <c r="BC6" s="411"/>
-      <c r="BD6" s="411"/>
-      <c r="BE6" s="411"/>
-      <c r="BF6" s="411"/>
-      <c r="BG6" s="411"/>
-      <c r="BH6" s="411"/>
-      <c r="BI6" s="411"/>
-      <c r="BJ6" s="411"/>
-      <c r="BK6" s="411"/>
-      <c r="BL6" s="412"/>
-      <c r="BM6" s="410" t="s">
+      <c r="AZ6" s="409"/>
+      <c r="BA6" s="409"/>
+      <c r="BB6" s="409"/>
+      <c r="BC6" s="409"/>
+      <c r="BD6" s="409"/>
+      <c r="BE6" s="409"/>
+      <c r="BF6" s="409"/>
+      <c r="BG6" s="409"/>
+      <c r="BH6" s="409"/>
+      <c r="BI6" s="409"/>
+      <c r="BJ6" s="409"/>
+      <c r="BK6" s="409"/>
+      <c r="BL6" s="410"/>
+      <c r="BM6" s="408" t="s">
         <v>64</v>
       </c>
-      <c r="BN6" s="411"/>
-      <c r="BO6" s="411"/>
-      <c r="BP6" s="411"/>
-      <c r="BQ6" s="412"/>
-      <c r="BR6" s="398" t="s">
+      <c r="BN6" s="409"/>
+      <c r="BO6" s="409"/>
+      <c r="BP6" s="409"/>
+      <c r="BQ6" s="410"/>
+      <c r="BR6" s="396" t="s">
         <v>65</v>
       </c>
-      <c r="BS6" s="398" t="s">
+      <c r="BS6" s="396" t="s">
         <v>66</v>
       </c>
-      <c r="BT6" s="396"/>
-      <c r="BU6" s="405"/>
-      <c r="BW6" s="408"/>
-      <c r="BX6" s="405"/>
-      <c r="BY6" s="420"/>
-      <c r="BZ6" s="420"/>
-      <c r="CA6" s="408"/>
-      <c r="CB6" s="396"/>
-      <c r="CC6" s="396"/>
-      <c r="CD6" s="396"/>
+      <c r="BT6" s="394"/>
+      <c r="BU6" s="403"/>
+      <c r="BW6" s="406"/>
+      <c r="BX6" s="403"/>
+      <c r="BY6" s="418"/>
+      <c r="BZ6" s="418"/>
+      <c r="CA6" s="406"/>
+      <c r="CB6" s="394"/>
+      <c r="CC6" s="394"/>
+      <c r="CD6" s="394"/>
       <c r="CH6" s="46"/>
       <c r="CI6" s="47"/>
     </row>
     <row r="7" spans="1:87" s="48" customFormat="1" ht="12">
-      <c r="A7" s="396"/>
-      <c r="B7" s="396"/>
-      <c r="C7" s="396"/>
-      <c r="D7" s="396"/>
-      <c r="E7" s="396"/>
-      <c r="F7" s="396"/>
-      <c r="G7" s="396"/>
-      <c r="H7" s="396"/>
-      <c r="I7" s="396"/>
-      <c r="J7" s="396"/>
-      <c r="K7" s="396"/>
-      <c r="L7" s="396"/>
-      <c r="M7" s="396"/>
-      <c r="N7" s="396"/>
-      <c r="O7" s="396"/>
-      <c r="P7" s="396"/>
-      <c r="Q7" s="396"/>
-      <c r="R7" s="396"/>
-      <c r="S7" s="396"/>
-      <c r="T7" s="396"/>
-      <c r="U7" s="396"/>
-      <c r="V7" s="406"/>
-      <c r="W7" s="432"/>
-      <c r="X7" s="396"/>
-      <c r="Y7" s="396"/>
-      <c r="Z7" s="396"/>
-      <c r="AA7" s="396"/>
-      <c r="AB7" s="396"/>
-      <c r="AC7" s="396"/>
-      <c r="AD7" s="396"/>
-      <c r="AE7" s="396"/>
-      <c r="AF7" s="396"/>
-      <c r="AG7" s="396"/>
-      <c r="AH7" s="396"/>
-      <c r="AI7" s="396"/>
-      <c r="AJ7" s="396"/>
-      <c r="AK7" s="405"/>
-      <c r="AL7" s="396"/>
-      <c r="AM7" s="396"/>
-      <c r="AN7" s="396"/>
-      <c r="AO7" s="396"/>
-      <c r="AP7" s="396"/>
-      <c r="AQ7" s="396"/>
-      <c r="AR7" s="396"/>
-      <c r="AS7" s="396"/>
-      <c r="AT7" s="396"/>
-      <c r="AU7" s="396"/>
-      <c r="AV7" s="396"/>
-      <c r="AW7" s="396"/>
-      <c r="AX7" s="396"/>
+      <c r="A7" s="394"/>
+      <c r="B7" s="394"/>
+      <c r="C7" s="394"/>
+      <c r="D7" s="394"/>
+      <c r="E7" s="394"/>
+      <c r="F7" s="394"/>
+      <c r="G7" s="394"/>
+      <c r="H7" s="394"/>
+      <c r="I7" s="394"/>
+      <c r="J7" s="394"/>
+      <c r="K7" s="394"/>
+      <c r="L7" s="394"/>
+      <c r="M7" s="394"/>
+      <c r="N7" s="394"/>
+      <c r="O7" s="394"/>
+      <c r="P7" s="394"/>
+      <c r="Q7" s="394"/>
+      <c r="R7" s="394"/>
+      <c r="S7" s="394"/>
+      <c r="T7" s="394"/>
+      <c r="U7" s="394"/>
+      <c r="V7" s="404"/>
+      <c r="W7" s="430"/>
+      <c r="X7" s="394"/>
+      <c r="Y7" s="394"/>
+      <c r="Z7" s="394"/>
+      <c r="AA7" s="394"/>
+      <c r="AB7" s="394"/>
+      <c r="AC7" s="394"/>
+      <c r="AD7" s="394"/>
+      <c r="AE7" s="394"/>
+      <c r="AF7" s="394"/>
+      <c r="AG7" s="394"/>
+      <c r="AH7" s="394"/>
+      <c r="AI7" s="394"/>
+      <c r="AJ7" s="394"/>
+      <c r="AK7" s="403"/>
+      <c r="AL7" s="394"/>
+      <c r="AM7" s="394"/>
+      <c r="AN7" s="394"/>
+      <c r="AO7" s="394"/>
+      <c r="AP7" s="394"/>
+      <c r="AQ7" s="394"/>
+      <c r="AR7" s="394"/>
+      <c r="AS7" s="394"/>
+      <c r="AT7" s="394"/>
+      <c r="AU7" s="394"/>
+      <c r="AV7" s="394"/>
+      <c r="AW7" s="394"/>
+      <c r="AX7" s="394"/>
       <c r="AY7" s="29" t="s">
         <v>67</v>
       </c>
@@ -12132,124 +12124,124 @@
       <c r="BA7" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="410" t="s">
+      <c r="BB7" s="408" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="402" t="s">
+      <c r="BC7" s="400" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="402" t="s">
+      <c r="BD7" s="400" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="423" t="s">
+      <c r="BE7" s="421" t="s">
         <v>73</v>
       </c>
-      <c r="BF7" s="402" t="s">
+      <c r="BF7" s="400" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="402" t="s">
+      <c r="BG7" s="400" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="402" t="s">
+      <c r="BH7" s="400" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="402" t="s">
+      <c r="BI7" s="400" t="s">
         <v>77</v>
       </c>
-      <c r="BJ7" s="402" t="s">
+      <c r="BJ7" s="400" t="s">
         <v>78</v>
       </c>
-      <c r="BK7" s="402" t="s">
+      <c r="BK7" s="400" t="s">
         <v>79</v>
       </c>
-      <c r="BL7" s="403" t="s">
+      <c r="BL7" s="401" t="s">
         <v>80</v>
       </c>
-      <c r="BM7" s="402" t="s">
+      <c r="BM7" s="400" t="s">
         <v>81</v>
       </c>
-      <c r="BN7" s="410" t="s">
+      <c r="BN7" s="408" t="s">
         <v>82</v>
       </c>
-      <c r="BO7" s="402" t="s">
+      <c r="BO7" s="400" t="s">
         <v>83</v>
       </c>
-      <c r="BP7" s="410" t="s">
+      <c r="BP7" s="408" t="s">
         <v>84</v>
       </c>
-      <c r="BQ7" s="410" t="s">
+      <c r="BQ7" s="408" t="s">
         <v>85</v>
       </c>
-      <c r="BR7" s="396"/>
-      <c r="BS7" s="396"/>
-      <c r="BT7" s="396"/>
-      <c r="BU7" s="405"/>
-      <c r="BW7" s="408"/>
-      <c r="BX7" s="421"/>
-      <c r="BY7" s="422"/>
-      <c r="BZ7" s="422"/>
-      <c r="CA7" s="409"/>
-      <c r="CB7" s="396"/>
-      <c r="CC7" s="396"/>
-      <c r="CD7" s="396"/>
+      <c r="BR7" s="394"/>
+      <c r="BS7" s="394"/>
+      <c r="BT7" s="394"/>
+      <c r="BU7" s="403"/>
+      <c r="BW7" s="406"/>
+      <c r="BX7" s="419"/>
+      <c r="BY7" s="420"/>
+      <c r="BZ7" s="420"/>
+      <c r="CA7" s="407"/>
+      <c r="CB7" s="394"/>
+      <c r="CC7" s="394"/>
+      <c r="CD7" s="394"/>
       <c r="CH7" s="46"/>
       <c r="CI7" s="47"/>
     </row>
     <row r="8" spans="1:87" s="48" customFormat="1" ht="12">
-      <c r="A8" s="399"/>
-      <c r="B8" s="399"/>
-      <c r="C8" s="399"/>
-      <c r="D8" s="399"/>
-      <c r="E8" s="399"/>
-      <c r="F8" s="399"/>
-      <c r="G8" s="399"/>
-      <c r="H8" s="399"/>
-      <c r="I8" s="399"/>
-      <c r="J8" s="399"/>
-      <c r="K8" s="399"/>
-      <c r="L8" s="399"/>
-      <c r="M8" s="399"/>
-      <c r="N8" s="399"/>
-      <c r="O8" s="399"/>
-      <c r="P8" s="399"/>
-      <c r="Q8" s="399"/>
-      <c r="R8" s="399"/>
-      <c r="S8" s="399"/>
-      <c r="T8" s="399"/>
-      <c r="U8" s="399"/>
+      <c r="A8" s="397"/>
+      <c r="B8" s="397"/>
+      <c r="C8" s="397"/>
+      <c r="D8" s="397"/>
+      <c r="E8" s="397"/>
+      <c r="F8" s="397"/>
+      <c r="G8" s="397"/>
+      <c r="H8" s="397"/>
+      <c r="I8" s="397"/>
+      <c r="J8" s="397"/>
+      <c r="K8" s="397"/>
+      <c r="L8" s="397"/>
+      <c r="M8" s="397"/>
+      <c r="N8" s="397"/>
+      <c r="O8" s="397"/>
+      <c r="P8" s="397"/>
+      <c r="Q8" s="397"/>
+      <c r="R8" s="397"/>
+      <c r="S8" s="397"/>
+      <c r="T8" s="397"/>
+      <c r="U8" s="397"/>
       <c r="V8" s="49" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="399"/>
-      <c r="Y8" s="399"/>
-      <c r="Z8" s="399"/>
-      <c r="AA8" s="399"/>
-      <c r="AB8" s="399"/>
-      <c r="AC8" s="399"/>
-      <c r="AD8" s="399"/>
-      <c r="AE8" s="399"/>
-      <c r="AF8" s="399"/>
-      <c r="AG8" s="399"/>
-      <c r="AH8" s="399"/>
-      <c r="AI8" s="399"/>
-      <c r="AJ8" s="399"/>
-      <c r="AK8" s="406"/>
-      <c r="AL8" s="399"/>
-      <c r="AM8" s="399"/>
-      <c r="AN8" s="399"/>
-      <c r="AO8" s="399"/>
-      <c r="AP8" s="399"/>
-      <c r="AQ8" s="399"/>
-      <c r="AR8" s="399"/>
-      <c r="AS8" s="399"/>
-      <c r="AT8" s="399"/>
-      <c r="AU8" s="399"/>
-      <c r="AV8" s="399"/>
-      <c r="AW8" s="399"/>
-      <c r="AX8" s="399"/>
+      <c r="X8" s="397"/>
+      <c r="Y8" s="397"/>
+      <c r="Z8" s="397"/>
+      <c r="AA8" s="397"/>
+      <c r="AB8" s="397"/>
+      <c r="AC8" s="397"/>
+      <c r="AD8" s="397"/>
+      <c r="AE8" s="397"/>
+      <c r="AF8" s="397"/>
+      <c r="AG8" s="397"/>
+      <c r="AH8" s="397"/>
+      <c r="AI8" s="397"/>
+      <c r="AJ8" s="397"/>
+      <c r="AK8" s="404"/>
+      <c r="AL8" s="397"/>
+      <c r="AM8" s="397"/>
+      <c r="AN8" s="397"/>
+      <c r="AO8" s="397"/>
+      <c r="AP8" s="397"/>
+      <c r="AQ8" s="397"/>
+      <c r="AR8" s="397"/>
+      <c r="AS8" s="397"/>
+      <c r="AT8" s="397"/>
+      <c r="AU8" s="397"/>
+      <c r="AV8" s="397"/>
+      <c r="AW8" s="397"/>
+      <c r="AX8" s="397"/>
       <c r="AY8" s="30" t="s">
         <v>88</v>
       </c>
@@ -12259,27 +12251,27 @@
       <c r="BA8" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="399"/>
-      <c r="BC8" s="399"/>
-      <c r="BD8" s="399"/>
-      <c r="BE8" s="399"/>
-      <c r="BF8" s="399"/>
-      <c r="BG8" s="399"/>
-      <c r="BH8" s="399"/>
-      <c r="BI8" s="399"/>
-      <c r="BJ8" s="399"/>
-      <c r="BK8" s="399"/>
-      <c r="BL8" s="399"/>
-      <c r="BM8" s="399"/>
-      <c r="BN8" s="399"/>
-      <c r="BO8" s="399"/>
-      <c r="BP8" s="399"/>
-      <c r="BQ8" s="399"/>
-      <c r="BR8" s="399"/>
-      <c r="BS8" s="399"/>
-      <c r="BT8" s="399"/>
-      <c r="BU8" s="406"/>
-      <c r="BW8" s="409"/>
+      <c r="BB8" s="397"/>
+      <c r="BC8" s="397"/>
+      <c r="BD8" s="397"/>
+      <c r="BE8" s="397"/>
+      <c r="BF8" s="397"/>
+      <c r="BG8" s="397"/>
+      <c r="BH8" s="397"/>
+      <c r="BI8" s="397"/>
+      <c r="BJ8" s="397"/>
+      <c r="BK8" s="397"/>
+      <c r="BL8" s="397"/>
+      <c r="BM8" s="397"/>
+      <c r="BN8" s="397"/>
+      <c r="BO8" s="397"/>
+      <c r="BP8" s="397"/>
+      <c r="BQ8" s="397"/>
+      <c r="BR8" s="397"/>
+      <c r="BS8" s="397"/>
+      <c r="BT8" s="397"/>
+      <c r="BU8" s="404"/>
+      <c r="BW8" s="407"/>
       <c r="BX8" s="23" t="s">
         <v>91</v>
       </c>
@@ -12292,9 +12284,9 @@
       <c r="CA8" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="397"/>
-      <c r="CC8" s="397"/>
-      <c r="CD8" s="397"/>
+      <c r="CB8" s="395"/>
+      <c r="CC8" s="395"/>
+      <c r="CD8" s="395"/>
       <c r="CE8" s="45"/>
       <c r="CF8" s="50"/>
       <c r="CH8" s="46"/>
@@ -15055,86 +15047,86 @@
       <c r="CB2" s="268"/>
     </row>
     <row r="3" spans="1:85" s="240" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="437"/>
-      <c r="B3" s="436"/>
-      <c r="C3" s="436"/>
-      <c r="D3" s="436"/>
-      <c r="E3" s="436"/>
-      <c r="F3" s="436"/>
-      <c r="G3" s="436"/>
-      <c r="H3" s="436"/>
-      <c r="I3" s="436"/>
-      <c r="J3" s="436"/>
-      <c r="K3" s="436"/>
-      <c r="L3" s="436"/>
-      <c r="M3" s="436"/>
-      <c r="N3" s="436"/>
-      <c r="O3" s="436"/>
-      <c r="P3" s="436"/>
-      <c r="Q3" s="436"/>
-      <c r="R3" s="436"/>
-      <c r="S3" s="436"/>
-      <c r="T3" s="436"/>
-      <c r="U3" s="436"/>
-      <c r="V3" s="436"/>
-      <c r="W3" s="436"/>
-      <c r="X3" s="436"/>
-      <c r="Y3" s="436"/>
-      <c r="Z3" s="436"/>
-      <c r="AA3" s="436"/>
-      <c r="AB3" s="436"/>
-      <c r="AC3" s="436"/>
-      <c r="AD3" s="436"/>
-      <c r="AE3" s="436"/>
-      <c r="AF3" s="436"/>
-      <c r="AG3" s="436"/>
-      <c r="AH3" s="436"/>
-      <c r="AI3" s="436"/>
-      <c r="AJ3" s="436"/>
-      <c r="AK3" s="436"/>
-      <c r="AL3" s="436"/>
-      <c r="AM3" s="436"/>
-      <c r="AN3" s="436"/>
-      <c r="AO3" s="436"/>
-      <c r="AP3" s="436"/>
-      <c r="AQ3" s="436"/>
-      <c r="AR3" s="436"/>
-      <c r="AS3" s="436"/>
-      <c r="AT3" s="436"/>
-      <c r="AU3" s="436"/>
-      <c r="AV3" s="436"/>
-      <c r="AW3" s="436"/>
-      <c r="AX3" s="436"/>
-      <c r="AY3" s="436"/>
-      <c r="AZ3" s="436"/>
-      <c r="BA3" s="436"/>
-      <c r="BB3" s="436"/>
-      <c r="BC3" s="436"/>
-      <c r="BD3" s="436"/>
-      <c r="BE3" s="436"/>
-      <c r="BF3" s="436"/>
-      <c r="BG3" s="436"/>
-      <c r="BH3" s="436"/>
-      <c r="BI3" s="436"/>
-      <c r="BJ3" s="436"/>
-      <c r="BK3" s="436"/>
-      <c r="BL3" s="436"/>
-      <c r="BM3" s="436"/>
-      <c r="BN3" s="436"/>
-      <c r="BO3" s="436"/>
-      <c r="BP3" s="436"/>
-      <c r="BQ3" s="436"/>
-      <c r="BR3" s="436"/>
-      <c r="BS3" s="436"/>
-      <c r="BT3" s="436"/>
-      <c r="BU3" s="435" t="s">
+      <c r="A3" s="435"/>
+      <c r="B3" s="434"/>
+      <c r="C3" s="434"/>
+      <c r="D3" s="434"/>
+      <c r="E3" s="434"/>
+      <c r="F3" s="434"/>
+      <c r="G3" s="434"/>
+      <c r="H3" s="434"/>
+      <c r="I3" s="434"/>
+      <c r="J3" s="434"/>
+      <c r="K3" s="434"/>
+      <c r="L3" s="434"/>
+      <c r="M3" s="434"/>
+      <c r="N3" s="434"/>
+      <c r="O3" s="434"/>
+      <c r="P3" s="434"/>
+      <c r="Q3" s="434"/>
+      <c r="R3" s="434"/>
+      <c r="S3" s="434"/>
+      <c r="T3" s="434"/>
+      <c r="U3" s="434"/>
+      <c r="V3" s="434"/>
+      <c r="W3" s="434"/>
+      <c r="X3" s="434"/>
+      <c r="Y3" s="434"/>
+      <c r="Z3" s="434"/>
+      <c r="AA3" s="434"/>
+      <c r="AB3" s="434"/>
+      <c r="AC3" s="434"/>
+      <c r="AD3" s="434"/>
+      <c r="AE3" s="434"/>
+      <c r="AF3" s="434"/>
+      <c r="AG3" s="434"/>
+      <c r="AH3" s="434"/>
+      <c r="AI3" s="434"/>
+      <c r="AJ3" s="434"/>
+      <c r="AK3" s="434"/>
+      <c r="AL3" s="434"/>
+      <c r="AM3" s="434"/>
+      <c r="AN3" s="434"/>
+      <c r="AO3" s="434"/>
+      <c r="AP3" s="434"/>
+      <c r="AQ3" s="434"/>
+      <c r="AR3" s="434"/>
+      <c r="AS3" s="434"/>
+      <c r="AT3" s="434"/>
+      <c r="AU3" s="434"/>
+      <c r="AV3" s="434"/>
+      <c r="AW3" s="434"/>
+      <c r="AX3" s="434"/>
+      <c r="AY3" s="434"/>
+      <c r="AZ3" s="434"/>
+      <c r="BA3" s="434"/>
+      <c r="BB3" s="434"/>
+      <c r="BC3" s="434"/>
+      <c r="BD3" s="434"/>
+      <c r="BE3" s="434"/>
+      <c r="BF3" s="434"/>
+      <c r="BG3" s="434"/>
+      <c r="BH3" s="434"/>
+      <c r="BI3" s="434"/>
+      <c r="BJ3" s="434"/>
+      <c r="BK3" s="434"/>
+      <c r="BL3" s="434"/>
+      <c r="BM3" s="434"/>
+      <c r="BN3" s="434"/>
+      <c r="BO3" s="434"/>
+      <c r="BP3" s="434"/>
+      <c r="BQ3" s="434"/>
+      <c r="BR3" s="434"/>
+      <c r="BS3" s="434"/>
+      <c r="BT3" s="434"/>
+      <c r="BU3" s="433" t="s">
         <v>2</v>
       </c>
-      <c r="BV3" s="436"/>
-      <c r="BW3" s="436"/>
-      <c r="BX3" s="436"/>
-      <c r="BY3" s="436"/>
-      <c r="BZ3" s="436"/>
+      <c r="BV3" s="434"/>
+      <c r="BW3" s="434"/>
+      <c r="BX3" s="434"/>
+      <c r="BY3" s="434"/>
+      <c r="BZ3" s="434"/>
       <c r="CA3" s="270"/>
       <c r="CB3" s="270"/>
     </row>
@@ -15210,12 +15202,12 @@
       <c r="BR4" s="271"/>
       <c r="BS4" s="271"/>
       <c r="BT4" s="271"/>
-      <c r="BU4" s="436"/>
-      <c r="BV4" s="436"/>
-      <c r="BW4" s="436"/>
-      <c r="BX4" s="436"/>
-      <c r="BY4" s="436"/>
-      <c r="BZ4" s="436"/>
+      <c r="BU4" s="434"/>
+      <c r="BV4" s="434"/>
+      <c r="BW4" s="434"/>
+      <c r="BX4" s="434"/>
+      <c r="BY4" s="434"/>
+      <c r="BZ4" s="434"/>
       <c r="CA4" s="270"/>
       <c r="CB4" s="270"/>
     </row>
@@ -15291,12 +15283,12 @@
       <c r="BR5" s="271"/>
       <c r="BS5" s="271"/>
       <c r="BT5" s="271"/>
-      <c r="BU5" s="436"/>
-      <c r="BV5" s="436"/>
-      <c r="BW5" s="436"/>
-      <c r="BX5" s="436"/>
-      <c r="BY5" s="436"/>
-      <c r="BZ5" s="436"/>
+      <c r="BU5" s="434"/>
+      <c r="BV5" s="434"/>
+      <c r="BW5" s="434"/>
+      <c r="BX5" s="434"/>
+      <c r="BY5" s="434"/>
+      <c r="BZ5" s="434"/>
       <c r="CA5" s="270"/>
       <c r="CB5" s="270"/>
     </row>
@@ -15372,12 +15364,12 @@
       <c r="BR6" s="273"/>
       <c r="BS6" s="273"/>
       <c r="BT6" s="273"/>
-      <c r="BU6" s="436"/>
-      <c r="BV6" s="436"/>
-      <c r="BW6" s="436"/>
-      <c r="BX6" s="436"/>
-      <c r="BY6" s="436"/>
-      <c r="BZ6" s="436"/>
+      <c r="BU6" s="434"/>
+      <c r="BV6" s="434"/>
+      <c r="BW6" s="434"/>
+      <c r="BX6" s="434"/>
+      <c r="BY6" s="434"/>
+      <c r="BZ6" s="434"/>
       <c r="CA6" s="270"/>
       <c r="CB6" s="270"/>
     </row>
@@ -15462,353 +15454,353 @@
       <c r="CA7" s="283"/>
       <c r="CB7" s="283"/>
     </row>
-    <row r="8" spans="1:85" s="451" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="444" t="s">
+    <row r="8" spans="1:85" s="448" customFormat="1" ht="19.25" customHeight="1">
+      <c r="A8" s="442" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="445" t="s">
+      <c r="B8" s="443" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="430" t="s">
+      <c r="C8" s="428" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="446" t="s">
+      <c r="D8" s="444" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="446" t="s">
+      <c r="E8" s="444" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="447" t="s">
+      <c r="F8" s="445" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="361" t="s">
+      <c r="G8" s="359" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="448" t="s">
+      <c r="H8" s="446" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="448" t="s">
+      <c r="I8" s="446" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="361" t="s">
+      <c r="J8" s="359" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="438" t="s">
+      <c r="K8" s="436" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="471"/>
-      <c r="M8" s="471"/>
-      <c r="N8" s="471"/>
-      <c r="O8" s="471"/>
-      <c r="P8" s="471"/>
-      <c r="Q8" s="471"/>
-      <c r="R8" s="471"/>
-      <c r="S8" s="471"/>
-      <c r="T8" s="471"/>
-      <c r="U8" s="471"/>
-      <c r="V8" s="471"/>
-      <c r="W8" s="471"/>
-      <c r="X8" s="471"/>
-      <c r="Y8" s="433" t="s">
+      <c r="L8" s="467"/>
+      <c r="M8" s="467"/>
+      <c r="N8" s="467"/>
+      <c r="O8" s="467"/>
+      <c r="P8" s="467"/>
+      <c r="Q8" s="467"/>
+      <c r="R8" s="467"/>
+      <c r="S8" s="467"/>
+      <c r="T8" s="467"/>
+      <c r="U8" s="467"/>
+      <c r="V8" s="467"/>
+      <c r="W8" s="467"/>
+      <c r="X8" s="467"/>
+      <c r="Y8" s="431" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="471"/>
-      <c r="AA8" s="471"/>
-      <c r="AB8" s="471"/>
-      <c r="AC8" s="471"/>
-      <c r="AD8" s="471"/>
-      <c r="AE8" s="471"/>
-      <c r="AF8" s="471"/>
-      <c r="AG8" s="471"/>
-      <c r="AH8" s="471"/>
-      <c r="AI8" s="471"/>
-      <c r="AJ8" s="471"/>
-      <c r="AK8" s="471"/>
-      <c r="AL8" s="471"/>
-      <c r="AM8" s="471"/>
-      <c r="AN8" s="471"/>
-      <c r="AO8" s="472"/>
-      <c r="AP8" s="361" t="s">
+      <c r="Z8" s="467"/>
+      <c r="AA8" s="467"/>
+      <c r="AB8" s="467"/>
+      <c r="AC8" s="467"/>
+      <c r="AD8" s="467"/>
+      <c r="AE8" s="467"/>
+      <c r="AF8" s="467"/>
+      <c r="AG8" s="467"/>
+      <c r="AH8" s="467"/>
+      <c r="AI8" s="467"/>
+      <c r="AJ8" s="467"/>
+      <c r="AK8" s="467"/>
+      <c r="AL8" s="467"/>
+      <c r="AM8" s="467"/>
+      <c r="AN8" s="467"/>
+      <c r="AO8" s="468"/>
+      <c r="AP8" s="359" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="361" t="s">
+      <c r="AQ8" s="359" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="361" t="s">
+      <c r="AR8" s="359" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="361" t="s">
+      <c r="AS8" s="359" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="361" t="s">
+      <c r="AT8" s="359" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="361" t="s">
+      <c r="AU8" s="359" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="349" t="s">
+      <c r="AV8" s="347" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="339" t="s">
+      <c r="AW8" s="337" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="349" t="s">
+      <c r="AX8" s="347" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="439" t="s">
+      <c r="AY8" s="437" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="471"/>
-      <c r="BA8" s="471"/>
-      <c r="BB8" s="471"/>
-      <c r="BC8" s="471"/>
-      <c r="BD8" s="471"/>
-      <c r="BE8" s="471"/>
-      <c r="BF8" s="471"/>
-      <c r="BG8" s="471"/>
-      <c r="BH8" s="471"/>
-      <c r="BI8" s="471"/>
-      <c r="BJ8" s="471"/>
-      <c r="BK8" s="471"/>
-      <c r="BL8" s="471"/>
-      <c r="BM8" s="471"/>
-      <c r="BN8" s="471"/>
-      <c r="BO8" s="471"/>
-      <c r="BP8" s="472"/>
-      <c r="BQ8" s="442" t="s">
+      <c r="AZ8" s="467"/>
+      <c r="BA8" s="467"/>
+      <c r="BB8" s="467"/>
+      <c r="BC8" s="467"/>
+      <c r="BD8" s="467"/>
+      <c r="BE8" s="467"/>
+      <c r="BF8" s="467"/>
+      <c r="BG8" s="467"/>
+      <c r="BH8" s="467"/>
+      <c r="BI8" s="467"/>
+      <c r="BJ8" s="467"/>
+      <c r="BK8" s="467"/>
+      <c r="BL8" s="467"/>
+      <c r="BM8" s="467"/>
+      <c r="BN8" s="467"/>
+      <c r="BO8" s="467"/>
+      <c r="BP8" s="468"/>
+      <c r="BQ8" s="440" t="s">
         <v>26</v>
       </c>
-      <c r="BR8" s="473"/>
-      <c r="BS8" s="430" t="s">
+      <c r="BR8" s="469"/>
+      <c r="BS8" s="428" t="s">
         <v>143</v>
       </c>
-      <c r="BT8" s="430" t="s">
+      <c r="BT8" s="428" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="391" t="s">
+      <c r="BU8" s="389" t="s">
         <v>29</v>
       </c>
-      <c r="BV8" s="440" t="s">
+      <c r="BV8" s="438" t="s">
         <v>30</v>
       </c>
-      <c r="BW8" s="476"/>
-      <c r="BX8" s="476"/>
-      <c r="BY8" s="477"/>
-      <c r="BZ8" s="395" t="s">
+      <c r="BW8" s="472"/>
+      <c r="BX8" s="472"/>
+      <c r="BY8" s="473"/>
+      <c r="BZ8" s="393" t="s">
         <v>31</v>
       </c>
-      <c r="CA8" s="395" t="s">
+      <c r="CA8" s="393" t="s">
         <v>32</v>
       </c>
-      <c r="CB8" s="450" t="s">
+      <c r="CB8" s="393" t="s">
         <v>33</v>
       </c>
-      <c r="CF8" s="452"/>
-      <c r="CG8" s="452"/>
+      <c r="CF8" s="449"/>
+      <c r="CG8" s="449"/>
     </row>
-    <row r="9" spans="1:85" s="451" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="453"/>
-      <c r="B9" s="453"/>
-      <c r="C9" s="453"/>
-      <c r="D9" s="453"/>
-      <c r="E9" s="453"/>
-      <c r="F9" s="453"/>
-      <c r="G9" s="340"/>
-      <c r="H9" s="453"/>
-      <c r="I9" s="453"/>
-      <c r="J9" s="340"/>
-      <c r="K9" s="454" t="s">
+    <row r="9" spans="1:85" s="448" customFormat="1" ht="19.25" customHeight="1">
+      <c r="A9" s="450"/>
+      <c r="B9" s="450"/>
+      <c r="C9" s="450"/>
+      <c r="D9" s="450"/>
+      <c r="E9" s="450"/>
+      <c r="F9" s="450"/>
+      <c r="G9" s="338"/>
+      <c r="H9" s="450"/>
+      <c r="I9" s="450"/>
+      <c r="J9" s="338"/>
+      <c r="K9" s="451" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="454" t="s">
+      <c r="L9" s="451" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="454" t="s">
+      <c r="M9" s="451" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="454" t="s">
+      <c r="N9" s="451" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="454" t="s">
+      <c r="O9" s="451" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="454" t="s">
+      <c r="P9" s="451" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="454" t="s">
+      <c r="Q9" s="451" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="454" t="s">
+      <c r="R9" s="451" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="454" t="s">
+      <c r="S9" s="451" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="454" t="s">
+      <c r="T9" s="451" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="454" t="s">
+      <c r="U9" s="451" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="455" t="s">
+      <c r="V9" s="452" t="s">
         <v>45</v>
       </c>
-      <c r="W9" s="449"/>
-      <c r="X9" s="454" t="s">
+      <c r="W9" s="447"/>
+      <c r="X9" s="451" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="456" t="s">
+      <c r="Y9" s="453" t="s">
         <v>47</v>
       </c>
-      <c r="Z9" s="456" t="s">
+      <c r="Z9" s="453" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="456" t="s">
+      <c r="AA9" s="453" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="456" t="s">
+      <c r="AB9" s="453" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="456" t="s">
+      <c r="AC9" s="453" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="456" t="s">
+      <c r="AD9" s="453" t="s">
         <v>144</v>
       </c>
-      <c r="AE9" s="456" t="s">
+      <c r="AE9" s="453" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="456" t="s">
+      <c r="AF9" s="453" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="456" t="s">
+      <c r="AG9" s="453" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="456" t="s">
+      <c r="AH9" s="453" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="456" t="s">
+      <c r="AI9" s="453" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="357" t="s">
+      <c r="AJ9" s="355" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="336" t="s">
+      <c r="AK9" s="334" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="339" t="s">
+      <c r="AL9" s="337" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="333" t="s">
+      <c r="AM9" s="331" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="349" t="s">
+      <c r="AN9" s="347" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="349" t="s">
+      <c r="AO9" s="347" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="340"/>
-      <c r="AQ9" s="340"/>
-      <c r="AR9" s="340"/>
-      <c r="AS9" s="340"/>
-      <c r="AT9" s="340"/>
-      <c r="AU9" s="340"/>
-      <c r="AV9" s="334"/>
-      <c r="AW9" s="340"/>
-      <c r="AX9" s="334"/>
-      <c r="AY9" s="434" t="s">
+      <c r="AP9" s="338"/>
+      <c r="AQ9" s="338"/>
+      <c r="AR9" s="338"/>
+      <c r="AS9" s="338"/>
+      <c r="AT9" s="338"/>
+      <c r="AU9" s="338"/>
+      <c r="AV9" s="332"/>
+      <c r="AW9" s="338"/>
+      <c r="AX9" s="332"/>
+      <c r="AY9" s="432" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="474"/>
-      <c r="BA9" s="474"/>
-      <c r="BB9" s="474"/>
-      <c r="BC9" s="474"/>
-      <c r="BD9" s="474"/>
-      <c r="BE9" s="474"/>
-      <c r="BF9" s="474"/>
-      <c r="BG9" s="474"/>
-      <c r="BH9" s="474"/>
-      <c r="BI9" s="474"/>
-      <c r="BJ9" s="475"/>
-      <c r="BK9" s="434" t="s">
+      <c r="AZ9" s="470"/>
+      <c r="BA9" s="470"/>
+      <c r="BB9" s="470"/>
+      <c r="BC9" s="470"/>
+      <c r="BD9" s="470"/>
+      <c r="BE9" s="470"/>
+      <c r="BF9" s="470"/>
+      <c r="BG9" s="470"/>
+      <c r="BH9" s="470"/>
+      <c r="BI9" s="470"/>
+      <c r="BJ9" s="471"/>
+      <c r="BK9" s="432" t="s">
         <v>64</v>
       </c>
-      <c r="BL9" s="474"/>
-      <c r="BM9" s="474"/>
-      <c r="BN9" s="474"/>
-      <c r="BO9" s="474"/>
-      <c r="BP9" s="475"/>
-      <c r="BQ9" s="457" t="s">
+      <c r="BL9" s="470"/>
+      <c r="BM9" s="470"/>
+      <c r="BN9" s="470"/>
+      <c r="BO9" s="470"/>
+      <c r="BP9" s="471"/>
+      <c r="BQ9" s="454" t="s">
         <v>65</v>
       </c>
-      <c r="BR9" s="457" t="s">
+      <c r="BR9" s="454" t="s">
         <v>66</v>
       </c>
-      <c r="BS9" s="453"/>
-      <c r="BT9" s="453"/>
-      <c r="BU9" s="392"/>
-      <c r="BV9" s="478"/>
-      <c r="BW9" s="441"/>
-      <c r="BX9" s="441"/>
-      <c r="BY9" s="479"/>
-      <c r="BZ9" s="453"/>
-      <c r="CA9" s="453"/>
-      <c r="CB9" s="340"/>
-      <c r="CF9" s="452"/>
-      <c r="CG9" s="452"/>
+      <c r="BS9" s="450"/>
+      <c r="BT9" s="450"/>
+      <c r="BU9" s="390"/>
+      <c r="BV9" s="474"/>
+      <c r="BW9" s="439"/>
+      <c r="BX9" s="439"/>
+      <c r="BY9" s="475"/>
+      <c r="BZ9" s="450"/>
+      <c r="CA9" s="450"/>
+      <c r="CB9" s="450"/>
+      <c r="CF9" s="449"/>
+      <c r="CG9" s="449"/>
     </row>
-    <row r="10" spans="1:85" s="465" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="453"/>
-      <c r="B10" s="453"/>
-      <c r="C10" s="453"/>
-      <c r="D10" s="453"/>
-      <c r="E10" s="453"/>
-      <c r="F10" s="453"/>
-      <c r="G10" s="340"/>
-      <c r="H10" s="453"/>
-      <c r="I10" s="453"/>
-      <c r="J10" s="340"/>
-      <c r="K10" s="453"/>
-      <c r="L10" s="453"/>
-      <c r="M10" s="453"/>
-      <c r="N10" s="453"/>
-      <c r="O10" s="453"/>
-      <c r="P10" s="453"/>
-      <c r="Q10" s="453"/>
-      <c r="R10" s="453"/>
-      <c r="S10" s="453"/>
-      <c r="T10" s="453"/>
-      <c r="U10" s="453"/>
-      <c r="V10" s="458"/>
-      <c r="W10" s="459"/>
-      <c r="X10" s="453"/>
-      <c r="Y10" s="453"/>
-      <c r="Z10" s="453"/>
-      <c r="AA10" s="453"/>
-      <c r="AB10" s="453"/>
-      <c r="AC10" s="453"/>
-      <c r="AD10" s="453"/>
-      <c r="AE10" s="453"/>
-      <c r="AF10" s="453"/>
-      <c r="AG10" s="453"/>
-      <c r="AH10" s="453"/>
-      <c r="AI10" s="453"/>
-      <c r="AJ10" s="340"/>
-      <c r="AK10" s="337"/>
-      <c r="AL10" s="340"/>
-      <c r="AM10" s="334"/>
-      <c r="AN10" s="334"/>
-      <c r="AO10" s="334"/>
-      <c r="AP10" s="340"/>
-      <c r="AQ10" s="340"/>
-      <c r="AR10" s="340"/>
-      <c r="AS10" s="340"/>
-      <c r="AT10" s="340"/>
-      <c r="AU10" s="340"/>
-      <c r="AV10" s="334"/>
-      <c r="AW10" s="340"/>
-      <c r="AX10" s="334"/>
+    <row r="10" spans="1:85" s="462" customFormat="1" ht="19.25" customHeight="1">
+      <c r="A10" s="450"/>
+      <c r="B10" s="450"/>
+      <c r="C10" s="450"/>
+      <c r="D10" s="450"/>
+      <c r="E10" s="450"/>
+      <c r="F10" s="450"/>
+      <c r="G10" s="338"/>
+      <c r="H10" s="450"/>
+      <c r="I10" s="450"/>
+      <c r="J10" s="338"/>
+      <c r="K10" s="450"/>
+      <c r="L10" s="450"/>
+      <c r="M10" s="450"/>
+      <c r="N10" s="450"/>
+      <c r="O10" s="450"/>
+      <c r="P10" s="450"/>
+      <c r="Q10" s="450"/>
+      <c r="R10" s="450"/>
+      <c r="S10" s="450"/>
+      <c r="T10" s="450"/>
+      <c r="U10" s="450"/>
+      <c r="V10" s="455"/>
+      <c r="W10" s="456"/>
+      <c r="X10" s="450"/>
+      <c r="Y10" s="450"/>
+      <c r="Z10" s="450"/>
+      <c r="AA10" s="450"/>
+      <c r="AB10" s="450"/>
+      <c r="AC10" s="450"/>
+      <c r="AD10" s="450"/>
+      <c r="AE10" s="450"/>
+      <c r="AF10" s="450"/>
+      <c r="AG10" s="450"/>
+      <c r="AH10" s="450"/>
+      <c r="AI10" s="450"/>
+      <c r="AJ10" s="338"/>
+      <c r="AK10" s="335"/>
+      <c r="AL10" s="338"/>
+      <c r="AM10" s="332"/>
+      <c r="AN10" s="332"/>
+      <c r="AO10" s="332"/>
+      <c r="AP10" s="338"/>
+      <c r="AQ10" s="338"/>
+      <c r="AR10" s="338"/>
+      <c r="AS10" s="338"/>
+      <c r="AT10" s="338"/>
+      <c r="AU10" s="338"/>
+      <c r="AV10" s="332"/>
+      <c r="AW10" s="338"/>
+      <c r="AX10" s="332"/>
       <c r="AY10" s="329" t="s">
         <v>67</v>
       </c>
@@ -15818,124 +15810,124 @@
       <c r="BA10" s="329" t="s">
         <v>69</v>
       </c>
-      <c r="BB10" s="460" t="s">
+      <c r="BB10" s="457" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="461" t="s">
+      <c r="BC10" s="458" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="461" t="s">
+      <c r="BD10" s="458" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="462" t="s">
+      <c r="BE10" s="459" t="s">
         <v>145</v>
       </c>
-      <c r="BF10" s="462" t="s">
+      <c r="BF10" s="459" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="462" t="s">
+      <c r="BG10" s="459" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="461" t="s">
+      <c r="BH10" s="458" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="462" t="s">
+      <c r="BI10" s="459" t="s">
         <v>79</v>
       </c>
-      <c r="BJ10" s="463" t="s">
+      <c r="BJ10" s="460" t="s">
         <v>80</v>
       </c>
-      <c r="BK10" s="461" t="s">
+      <c r="BK10" s="458" t="s">
         <v>81</v>
       </c>
-      <c r="BL10" s="464" t="s">
+      <c r="BL10" s="461" t="s">
         <v>82</v>
       </c>
-      <c r="BM10" s="461" t="s">
+      <c r="BM10" s="458" t="s">
         <v>83</v>
       </c>
-      <c r="BN10" s="464" t="s">
+      <c r="BN10" s="461" t="s">
         <v>84</v>
       </c>
-      <c r="BO10" s="464" t="s">
+      <c r="BO10" s="461" t="s">
         <v>146</v>
       </c>
-      <c r="BP10" s="430" t="s">
+      <c r="BP10" s="428" t="s">
         <v>85</v>
       </c>
-      <c r="BQ10" s="453"/>
-      <c r="BR10" s="453"/>
-      <c r="BS10" s="453"/>
-      <c r="BT10" s="453"/>
-      <c r="BU10" s="392"/>
-      <c r="BV10" s="480"/>
-      <c r="BW10" s="481"/>
-      <c r="BX10" s="481"/>
-      <c r="BY10" s="482"/>
-      <c r="BZ10" s="453"/>
-      <c r="CA10" s="453"/>
-      <c r="CB10" s="340"/>
+      <c r="BQ10" s="450"/>
+      <c r="BR10" s="450"/>
+      <c r="BS10" s="450"/>
+      <c r="BT10" s="450"/>
+      <c r="BU10" s="390"/>
+      <c r="BV10" s="476"/>
+      <c r="BW10" s="477"/>
+      <c r="BX10" s="477"/>
+      <c r="BY10" s="478"/>
+      <c r="BZ10" s="450"/>
+      <c r="CA10" s="450"/>
+      <c r="CB10" s="450"/>
       <c r="CC10" s="228" t="s">
         <v>3</v>
       </c>
-      <c r="CF10" s="452"/>
-      <c r="CG10" s="452"/>
+      <c r="CF10" s="449"/>
+      <c r="CG10" s="449"/>
     </row>
-    <row r="11" spans="1:85" s="465" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="466"/>
-      <c r="B11" s="466"/>
-      <c r="C11" s="466"/>
-      <c r="D11" s="466"/>
-      <c r="E11" s="466"/>
-      <c r="F11" s="466"/>
-      <c r="G11" s="341"/>
-      <c r="H11" s="466"/>
-      <c r="I11" s="466"/>
-      <c r="J11" s="341"/>
-      <c r="K11" s="466"/>
-      <c r="L11" s="466"/>
-      <c r="M11" s="466"/>
-      <c r="N11" s="466"/>
-      <c r="O11" s="466"/>
-      <c r="P11" s="466"/>
-      <c r="Q11" s="466"/>
-      <c r="R11" s="466"/>
-      <c r="S11" s="466"/>
-      <c r="T11" s="466"/>
-      <c r="U11" s="466"/>
-      <c r="V11" s="467" t="s">
+    <row r="11" spans="1:85" s="462" customFormat="1" ht="38.25" customHeight="1">
+      <c r="A11" s="463"/>
+      <c r="B11" s="463"/>
+      <c r="C11" s="463"/>
+      <c r="D11" s="463"/>
+      <c r="E11" s="463"/>
+      <c r="F11" s="463"/>
+      <c r="G11" s="339"/>
+      <c r="H11" s="463"/>
+      <c r="I11" s="463"/>
+      <c r="J11" s="339"/>
+      <c r="K11" s="463"/>
+      <c r="L11" s="463"/>
+      <c r="M11" s="463"/>
+      <c r="N11" s="463"/>
+      <c r="O11" s="463"/>
+      <c r="P11" s="463"/>
+      <c r="Q11" s="463"/>
+      <c r="R11" s="463"/>
+      <c r="S11" s="463"/>
+      <c r="T11" s="463"/>
+      <c r="U11" s="463"/>
+      <c r="V11" s="464" t="s">
         <v>86</v>
       </c>
-      <c r="W11" s="467" t="s">
+      <c r="W11" s="464" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="466"/>
-      <c r="Y11" s="466"/>
-      <c r="Z11" s="466"/>
-      <c r="AA11" s="466"/>
-      <c r="AB11" s="466"/>
-      <c r="AC11" s="466"/>
-      <c r="AD11" s="466"/>
-      <c r="AE11" s="466"/>
-      <c r="AF11" s="466"/>
-      <c r="AG11" s="466"/>
-      <c r="AH11" s="466"/>
-      <c r="AI11" s="466"/>
-      <c r="AJ11" s="341"/>
-      <c r="AK11" s="338"/>
-      <c r="AL11" s="341"/>
-      <c r="AM11" s="335"/>
-      <c r="AN11" s="335"/>
-      <c r="AO11" s="335"/>
-      <c r="AP11" s="341"/>
-      <c r="AQ11" s="341"/>
-      <c r="AR11" s="341"/>
-      <c r="AS11" s="341"/>
-      <c r="AT11" s="341"/>
-      <c r="AU11" s="341"/>
-      <c r="AV11" s="335"/>
-      <c r="AW11" s="341"/>
-      <c r="AX11" s="335"/>
+      <c r="X11" s="463"/>
+      <c r="Y11" s="463"/>
+      <c r="Z11" s="463"/>
+      <c r="AA11" s="463"/>
+      <c r="AB11" s="463"/>
+      <c r="AC11" s="463"/>
+      <c r="AD11" s="463"/>
+      <c r="AE11" s="463"/>
+      <c r="AF11" s="463"/>
+      <c r="AG11" s="463"/>
+      <c r="AH11" s="463"/>
+      <c r="AI11" s="463"/>
+      <c r="AJ11" s="339"/>
+      <c r="AK11" s="336"/>
+      <c r="AL11" s="339"/>
+      <c r="AM11" s="333"/>
+      <c r="AN11" s="333"/>
+      <c r="AO11" s="333"/>
+      <c r="AP11" s="339"/>
+      <c r="AQ11" s="339"/>
+      <c r="AR11" s="339"/>
+      <c r="AS11" s="339"/>
+      <c r="AT11" s="339"/>
+      <c r="AU11" s="339"/>
+      <c r="AV11" s="333"/>
+      <c r="AW11" s="339"/>
+      <c r="AX11" s="333"/>
       <c r="AY11" s="229" t="s">
         <v>88</v>
       </c>
@@ -15945,26 +15937,26 @@
       <c r="BA11" s="229" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="466"/>
-      <c r="BC11" s="341"/>
-      <c r="BD11" s="341"/>
-      <c r="BE11" s="466"/>
-      <c r="BF11" s="466"/>
-      <c r="BG11" s="466"/>
-      <c r="BH11" s="341"/>
-      <c r="BI11" s="466"/>
-      <c r="BJ11" s="466"/>
-      <c r="BK11" s="341"/>
-      <c r="BL11" s="341"/>
-      <c r="BM11" s="341"/>
-      <c r="BN11" s="341"/>
-      <c r="BO11" s="341"/>
-      <c r="BP11" s="466"/>
-      <c r="BQ11" s="466"/>
-      <c r="BR11" s="466"/>
-      <c r="BS11" s="466"/>
-      <c r="BT11" s="466"/>
-      <c r="BU11" s="393"/>
+      <c r="BB11" s="463"/>
+      <c r="BC11" s="339"/>
+      <c r="BD11" s="339"/>
+      <c r="BE11" s="463"/>
+      <c r="BF11" s="463"/>
+      <c r="BG11" s="463"/>
+      <c r="BH11" s="339"/>
+      <c r="BI11" s="463"/>
+      <c r="BJ11" s="463"/>
+      <c r="BK11" s="339"/>
+      <c r="BL11" s="339"/>
+      <c r="BM11" s="339"/>
+      <c r="BN11" s="339"/>
+      <c r="BO11" s="339"/>
+      <c r="BP11" s="463"/>
+      <c r="BQ11" s="463"/>
+      <c r="BR11" s="463"/>
+      <c r="BS11" s="463"/>
+      <c r="BT11" s="463"/>
+      <c r="BU11" s="391"/>
       <c r="BV11" s="237" t="s">
         <v>91</v>
       </c>
@@ -15977,15 +15969,15 @@
       <c r="BY11" s="238" t="s">
         <v>94</v>
       </c>
-      <c r="BZ11" s="468"/>
-      <c r="CA11" s="468"/>
-      <c r="CB11" s="469"/>
+      <c r="BZ11" s="465"/>
+      <c r="CA11" s="465"/>
+      <c r="CB11" s="465"/>
       <c r="CC11" s="227">
         <v>25</v>
       </c>
-      <c r="CD11" s="470"/>
-      <c r="CF11" s="452"/>
-      <c r="CG11" s="452"/>
+      <c r="CD11" s="466"/>
+      <c r="CF11" s="449"/>
+      <c r="CG11" s="449"/>
     </row>
     <row r="12" spans="1:85" s="278" customFormat="1" ht="15" customHeight="1">
       <c r="A12" s="284">
@@ -18636,87 +18628,87 @@
       <c r="CD2" s="41"/>
     </row>
     <row r="3" spans="1:87" s="43" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="424"/>
-      <c r="B3" s="415"/>
-      <c r="C3" s="415"/>
-      <c r="D3" s="415"/>
-      <c r="E3" s="415"/>
-      <c r="F3" s="415"/>
-      <c r="G3" s="415"/>
-      <c r="H3" s="415"/>
-      <c r="I3" s="415"/>
-      <c r="J3" s="415"/>
-      <c r="K3" s="415"/>
-      <c r="L3" s="415"/>
-      <c r="M3" s="415"/>
-      <c r="N3" s="415"/>
-      <c r="O3" s="415"/>
-      <c r="P3" s="415"/>
-      <c r="Q3" s="415"/>
-      <c r="R3" s="415"/>
-      <c r="S3" s="415"/>
-      <c r="T3" s="415"/>
-      <c r="U3" s="415"/>
-      <c r="V3" s="415"/>
-      <c r="W3" s="415"/>
-      <c r="X3" s="415"/>
-      <c r="Y3" s="415"/>
-      <c r="Z3" s="415"/>
-      <c r="AA3" s="415"/>
-      <c r="AB3" s="415"/>
-      <c r="AC3" s="415"/>
-      <c r="AD3" s="415"/>
-      <c r="AE3" s="415"/>
-      <c r="AF3" s="415"/>
-      <c r="AG3" s="415"/>
-      <c r="AH3" s="415"/>
-      <c r="AI3" s="415"/>
-      <c r="AJ3" s="415"/>
-      <c r="AK3" s="415"/>
-      <c r="AL3" s="415"/>
-      <c r="AM3" s="415"/>
-      <c r="AN3" s="415"/>
-      <c r="AO3" s="415"/>
-      <c r="AP3" s="415"/>
-      <c r="AQ3" s="415"/>
-      <c r="AR3" s="415"/>
-      <c r="AS3" s="415"/>
-      <c r="AT3" s="415"/>
-      <c r="AU3" s="415"/>
-      <c r="AV3" s="415"/>
-      <c r="AW3" s="415"/>
-      <c r="AX3" s="415"/>
-      <c r="AY3" s="415"/>
-      <c r="AZ3" s="415"/>
-      <c r="BA3" s="415"/>
-      <c r="BB3" s="415"/>
-      <c r="BC3" s="415"/>
-      <c r="BD3" s="415"/>
-      <c r="BE3" s="415"/>
-      <c r="BF3" s="415"/>
-      <c r="BG3" s="415"/>
-      <c r="BH3" s="415"/>
-      <c r="BI3" s="415"/>
-      <c r="BJ3" s="415"/>
-      <c r="BK3" s="415"/>
-      <c r="BL3" s="415"/>
-      <c r="BM3" s="415"/>
-      <c r="BN3" s="415"/>
-      <c r="BO3" s="415"/>
-      <c r="BP3" s="415"/>
-      <c r="BQ3" s="415"/>
-      <c r="BR3" s="415"/>
-      <c r="BS3" s="415"/>
-      <c r="BT3" s="415"/>
-      <c r="BU3" s="415"/>
-      <c r="BW3" s="414" t="s">
+      <c r="A3" s="422"/>
+      <c r="B3" s="413"/>
+      <c r="C3" s="413"/>
+      <c r="D3" s="413"/>
+      <c r="E3" s="413"/>
+      <c r="F3" s="413"/>
+      <c r="G3" s="413"/>
+      <c r="H3" s="413"/>
+      <c r="I3" s="413"/>
+      <c r="J3" s="413"/>
+      <c r="K3" s="413"/>
+      <c r="L3" s="413"/>
+      <c r="M3" s="413"/>
+      <c r="N3" s="413"/>
+      <c r="O3" s="413"/>
+      <c r="P3" s="413"/>
+      <c r="Q3" s="413"/>
+      <c r="R3" s="413"/>
+      <c r="S3" s="413"/>
+      <c r="T3" s="413"/>
+      <c r="U3" s="413"/>
+      <c r="V3" s="413"/>
+      <c r="W3" s="413"/>
+      <c r="X3" s="413"/>
+      <c r="Y3" s="413"/>
+      <c r="Z3" s="413"/>
+      <c r="AA3" s="413"/>
+      <c r="AB3" s="413"/>
+      <c r="AC3" s="413"/>
+      <c r="AD3" s="413"/>
+      <c r="AE3" s="413"/>
+      <c r="AF3" s="413"/>
+      <c r="AG3" s="413"/>
+      <c r="AH3" s="413"/>
+      <c r="AI3" s="413"/>
+      <c r="AJ3" s="413"/>
+      <c r="AK3" s="413"/>
+      <c r="AL3" s="413"/>
+      <c r="AM3" s="413"/>
+      <c r="AN3" s="413"/>
+      <c r="AO3" s="413"/>
+      <c r="AP3" s="413"/>
+      <c r="AQ3" s="413"/>
+      <c r="AR3" s="413"/>
+      <c r="AS3" s="413"/>
+      <c r="AT3" s="413"/>
+      <c r="AU3" s="413"/>
+      <c r="AV3" s="413"/>
+      <c r="AW3" s="413"/>
+      <c r="AX3" s="413"/>
+      <c r="AY3" s="413"/>
+      <c r="AZ3" s="413"/>
+      <c r="BA3" s="413"/>
+      <c r="BB3" s="413"/>
+      <c r="BC3" s="413"/>
+      <c r="BD3" s="413"/>
+      <c r="BE3" s="413"/>
+      <c r="BF3" s="413"/>
+      <c r="BG3" s="413"/>
+      <c r="BH3" s="413"/>
+      <c r="BI3" s="413"/>
+      <c r="BJ3" s="413"/>
+      <c r="BK3" s="413"/>
+      <c r="BL3" s="413"/>
+      <c r="BM3" s="413"/>
+      <c r="BN3" s="413"/>
+      <c r="BO3" s="413"/>
+      <c r="BP3" s="413"/>
+      <c r="BQ3" s="413"/>
+      <c r="BR3" s="413"/>
+      <c r="BS3" s="413"/>
+      <c r="BT3" s="413"/>
+      <c r="BU3" s="413"/>
+      <c r="BW3" s="412" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="415"/>
-      <c r="BY3" s="415"/>
-      <c r="BZ3" s="415"/>
-      <c r="CA3" s="415"/>
-      <c r="CB3" s="415"/>
+      <c r="BX3" s="413"/>
+      <c r="BY3" s="413"/>
+      <c r="BZ3" s="413"/>
+      <c r="CA3" s="413"/>
+      <c r="CB3" s="413"/>
       <c r="CC3" s="42"/>
       <c r="CD3" s="42"/>
       <c r="CE3" s="43" t="s">
@@ -18799,366 +18791,366 @@
       <c r="BS4" s="44"/>
       <c r="BT4" s="44"/>
       <c r="BU4" s="44"/>
-      <c r="BW4" s="415"/>
-      <c r="BX4" s="415"/>
-      <c r="BY4" s="415"/>
-      <c r="BZ4" s="415"/>
-      <c r="CA4" s="415"/>
-      <c r="CB4" s="415"/>
+      <c r="BW4" s="413"/>
+      <c r="BX4" s="413"/>
+      <c r="BY4" s="413"/>
+      <c r="BZ4" s="413"/>
+      <c r="CA4" s="413"/>
+      <c r="CB4" s="413"/>
       <c r="CC4" s="42"/>
       <c r="CD4" s="42"/>
     </row>
     <row r="5" spans="1:87" s="45" customFormat="1">
-      <c r="A5" s="427" t="s">
+      <c r="A5" s="425" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="426" t="s">
+      <c r="B5" s="424" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="400" t="s">
+      <c r="C5" s="398" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="425" t="s">
+      <c r="D5" s="423" t="s">
         <v>141</v>
       </c>
-      <c r="E5" s="425" t="s">
+      <c r="E5" s="423" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="443" t="s">
+      <c r="F5" s="441" t="s">
         <v>142</v>
       </c>
-      <c r="G5" s="400" t="s">
+      <c r="G5" s="398" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="349" t="s">
+      <c r="H5" s="347" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="349" t="s">
+      <c r="I5" s="347" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="400" t="s">
+      <c r="J5" s="398" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="429" t="s">
+      <c r="K5" s="427" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="411"/>
-      <c r="M5" s="411"/>
-      <c r="N5" s="411"/>
-      <c r="O5" s="411"/>
-      <c r="P5" s="411"/>
-      <c r="Q5" s="411"/>
-      <c r="R5" s="411"/>
-      <c r="S5" s="411"/>
-      <c r="T5" s="411"/>
-      <c r="U5" s="411"/>
-      <c r="V5" s="411"/>
-      <c r="W5" s="411"/>
-      <c r="X5" s="411"/>
-      <c r="Y5" s="400" t="s">
+      <c r="L5" s="409"/>
+      <c r="M5" s="409"/>
+      <c r="N5" s="409"/>
+      <c r="O5" s="409"/>
+      <c r="P5" s="409"/>
+      <c r="Q5" s="409"/>
+      <c r="R5" s="409"/>
+      <c r="S5" s="409"/>
+      <c r="T5" s="409"/>
+      <c r="U5" s="409"/>
+      <c r="V5" s="409"/>
+      <c r="W5" s="409"/>
+      <c r="X5" s="409"/>
+      <c r="Y5" s="398" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="411"/>
-      <c r="AA5" s="411"/>
-      <c r="AB5" s="411"/>
-      <c r="AC5" s="411"/>
-      <c r="AD5" s="411"/>
-      <c r="AE5" s="411"/>
-      <c r="AF5" s="411"/>
-      <c r="AG5" s="411"/>
-      <c r="AH5" s="411"/>
-      <c r="AI5" s="411"/>
-      <c r="AJ5" s="411"/>
-      <c r="AK5" s="411"/>
-      <c r="AL5" s="411"/>
-      <c r="AM5" s="411"/>
-      <c r="AN5" s="411"/>
-      <c r="AO5" s="412"/>
-      <c r="AP5" s="400" t="s">
+      <c r="Z5" s="409"/>
+      <c r="AA5" s="409"/>
+      <c r="AB5" s="409"/>
+      <c r="AC5" s="409"/>
+      <c r="AD5" s="409"/>
+      <c r="AE5" s="409"/>
+      <c r="AF5" s="409"/>
+      <c r="AG5" s="409"/>
+      <c r="AH5" s="409"/>
+      <c r="AI5" s="409"/>
+      <c r="AJ5" s="409"/>
+      <c r="AK5" s="409"/>
+      <c r="AL5" s="409"/>
+      <c r="AM5" s="409"/>
+      <c r="AN5" s="409"/>
+      <c r="AO5" s="410"/>
+      <c r="AP5" s="398" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="400" t="s">
+      <c r="AQ5" s="398" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="400" t="s">
+      <c r="AR5" s="398" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="400" t="s">
+      <c r="AS5" s="398" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="400" t="s">
+      <c r="AT5" s="398" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="400" t="s">
+      <c r="AU5" s="398" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="400" t="s">
+      <c r="AV5" s="398" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="400" t="s">
+      <c r="AW5" s="398" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="400" t="s">
+      <c r="AX5" s="398" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="410" t="s">
+      <c r="AY5" s="408" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="411"/>
-      <c r="BA5" s="411"/>
-      <c r="BB5" s="411"/>
-      <c r="BC5" s="411"/>
-      <c r="BD5" s="411"/>
-      <c r="BE5" s="411"/>
-      <c r="BF5" s="411"/>
-      <c r="BG5" s="411"/>
-      <c r="BH5" s="411"/>
-      <c r="BI5" s="411"/>
-      <c r="BJ5" s="411"/>
-      <c r="BK5" s="411"/>
-      <c r="BL5" s="411"/>
-      <c r="BM5" s="411"/>
-      <c r="BN5" s="411"/>
-      <c r="BO5" s="411"/>
-      <c r="BP5" s="412"/>
-      <c r="BQ5" s="416" t="s">
+      <c r="AZ5" s="409"/>
+      <c r="BA5" s="409"/>
+      <c r="BB5" s="409"/>
+      <c r="BC5" s="409"/>
+      <c r="BD5" s="409"/>
+      <c r="BE5" s="409"/>
+      <c r="BF5" s="409"/>
+      <c r="BG5" s="409"/>
+      <c r="BH5" s="409"/>
+      <c r="BI5" s="409"/>
+      <c r="BJ5" s="409"/>
+      <c r="BK5" s="409"/>
+      <c r="BL5" s="409"/>
+      <c r="BM5" s="409"/>
+      <c r="BN5" s="409"/>
+      <c r="BO5" s="409"/>
+      <c r="BP5" s="410"/>
+      <c r="BQ5" s="414" t="s">
         <v>26</v>
       </c>
-      <c r="BR5" s="417"/>
-      <c r="BS5" s="410" t="s">
+      <c r="BR5" s="415"/>
+      <c r="BS5" s="408" t="s">
         <v>143</v>
       </c>
-      <c r="BT5" s="410" t="s">
+      <c r="BT5" s="408" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="404" t="s">
+      <c r="BU5" s="402" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="407" t="s">
+      <c r="BW5" s="405" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="418" t="s">
+      <c r="BX5" s="416" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="419"/>
-      <c r="BZ5" s="419"/>
-      <c r="CA5" s="417"/>
-      <c r="CB5" s="413" t="s">
+      <c r="BY5" s="417"/>
+      <c r="BZ5" s="417"/>
+      <c r="CA5" s="415"/>
+      <c r="CB5" s="411" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="395" t="s">
+      <c r="CC5" s="393" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="395" t="s">
+      <c r="CD5" s="393" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="46"/>
       <c r="CI5" s="47"/>
     </row>
     <row r="6" spans="1:87" s="45" customFormat="1">
-      <c r="A6" s="396"/>
-      <c r="B6" s="396"/>
-      <c r="C6" s="396"/>
-      <c r="D6" s="396"/>
-      <c r="E6" s="396"/>
-      <c r="F6" s="396"/>
-      <c r="G6" s="396"/>
-      <c r="H6" s="396"/>
-      <c r="I6" s="396"/>
-      <c r="J6" s="396"/>
-      <c r="K6" s="401" t="s">
+      <c r="A6" s="394"/>
+      <c r="B6" s="394"/>
+      <c r="C6" s="394"/>
+      <c r="D6" s="394"/>
+      <c r="E6" s="394"/>
+      <c r="F6" s="394"/>
+      <c r="G6" s="394"/>
+      <c r="H6" s="394"/>
+      <c r="I6" s="394"/>
+      <c r="J6" s="394"/>
+      <c r="K6" s="399" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="401" t="s">
+      <c r="L6" s="399" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="401" t="s">
+      <c r="M6" s="399" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="401" t="s">
+      <c r="N6" s="399" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="401" t="s">
+      <c r="O6" s="399" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="401" t="s">
+      <c r="P6" s="399" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="401" t="s">
+      <c r="Q6" s="399" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="401" t="s">
+      <c r="R6" s="399" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="401" t="s">
+      <c r="S6" s="399" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="401" t="s">
+      <c r="T6" s="399" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="401" t="s">
+      <c r="U6" s="399" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="431" t="s">
+      <c r="V6" s="429" t="s">
         <v>45</v>
       </c>
-      <c r="W6" s="417"/>
-      <c r="X6" s="401" t="s">
+      <c r="W6" s="415"/>
+      <c r="X6" s="399" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="400" t="s">
+      <c r="Y6" s="398" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="400" t="s">
+      <c r="Z6" s="398" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="400" t="s">
+      <c r="AA6" s="398" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="400" t="s">
+      <c r="AB6" s="398" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="349" t="s">
+      <c r="AC6" s="347" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="349" t="s">
+      <c r="AD6" s="347" t="s">
         <v>144</v>
       </c>
-      <c r="AE6" s="349" t="s">
+      <c r="AE6" s="347" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="349" t="s">
+      <c r="AF6" s="347" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="400" t="s">
+      <c r="AG6" s="398" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="349" t="s">
+      <c r="AH6" s="347" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="349" t="s">
+      <c r="AI6" s="347" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="400" t="s">
+      <c r="AJ6" s="398" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="428" t="s">
+      <c r="AK6" s="426" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="400" t="s">
+      <c r="AL6" s="398" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="400" t="s">
+      <c r="AM6" s="398" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="430" t="s">
+      <c r="AN6" s="428" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="400" t="s">
+      <c r="AO6" s="398" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="396"/>
-      <c r="AQ6" s="396"/>
-      <c r="AR6" s="396"/>
-      <c r="AS6" s="396"/>
-      <c r="AT6" s="396"/>
-      <c r="AU6" s="396"/>
-      <c r="AV6" s="396"/>
-      <c r="AW6" s="396"/>
-      <c r="AX6" s="396"/>
-      <c r="AY6" s="410" t="s">
+      <c r="AP6" s="394"/>
+      <c r="AQ6" s="394"/>
+      <c r="AR6" s="394"/>
+      <c r="AS6" s="394"/>
+      <c r="AT6" s="394"/>
+      <c r="AU6" s="394"/>
+      <c r="AV6" s="394"/>
+      <c r="AW6" s="394"/>
+      <c r="AX6" s="394"/>
+      <c r="AY6" s="408" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="411"/>
-      <c r="BA6" s="411"/>
-      <c r="BB6" s="411"/>
-      <c r="BC6" s="411"/>
-      <c r="BD6" s="411"/>
-      <c r="BE6" s="411"/>
-      <c r="BF6" s="411"/>
-      <c r="BG6" s="411"/>
-      <c r="BH6" s="411"/>
-      <c r="BI6" s="411"/>
-      <c r="BJ6" s="412"/>
-      <c r="BK6" s="410" t="s">
+      <c r="AZ6" s="409"/>
+      <c r="BA6" s="409"/>
+      <c r="BB6" s="409"/>
+      <c r="BC6" s="409"/>
+      <c r="BD6" s="409"/>
+      <c r="BE6" s="409"/>
+      <c r="BF6" s="409"/>
+      <c r="BG6" s="409"/>
+      <c r="BH6" s="409"/>
+      <c r="BI6" s="409"/>
+      <c r="BJ6" s="410"/>
+      <c r="BK6" s="408" t="s">
         <v>64</v>
       </c>
-      <c r="BL6" s="411"/>
-      <c r="BM6" s="411"/>
-      <c r="BN6" s="411"/>
-      <c r="BO6" s="411"/>
-      <c r="BP6" s="412"/>
-      <c r="BQ6" s="398" t="s">
+      <c r="BL6" s="409"/>
+      <c r="BM6" s="409"/>
+      <c r="BN6" s="409"/>
+      <c r="BO6" s="409"/>
+      <c r="BP6" s="410"/>
+      <c r="BQ6" s="396" t="s">
         <v>65</v>
       </c>
-      <c r="BR6" s="398" t="s">
+      <c r="BR6" s="396" t="s">
         <v>66</v>
       </c>
-      <c r="BS6" s="396"/>
-      <c r="BT6" s="396"/>
-      <c r="BU6" s="405"/>
-      <c r="BW6" s="408"/>
-      <c r="BX6" s="405"/>
-      <c r="BY6" s="420"/>
-      <c r="BZ6" s="420"/>
-      <c r="CA6" s="408"/>
-      <c r="CB6" s="396"/>
-      <c r="CC6" s="396"/>
-      <c r="CD6" s="396"/>
+      <c r="BS6" s="394"/>
+      <c r="BT6" s="394"/>
+      <c r="BU6" s="403"/>
+      <c r="BW6" s="406"/>
+      <c r="BX6" s="403"/>
+      <c r="BY6" s="418"/>
+      <c r="BZ6" s="418"/>
+      <c r="CA6" s="406"/>
+      <c r="CB6" s="394"/>
+      <c r="CC6" s="394"/>
+      <c r="CD6" s="394"/>
       <c r="CH6" s="46"/>
       <c r="CI6" s="47"/>
     </row>
     <row r="7" spans="1:87" s="45" customFormat="1" ht="12">
-      <c r="A7" s="396"/>
-      <c r="B7" s="396"/>
-      <c r="C7" s="396"/>
-      <c r="D7" s="396"/>
-      <c r="E7" s="396"/>
-      <c r="F7" s="396"/>
-      <c r="G7" s="396"/>
-      <c r="H7" s="396"/>
-      <c r="I7" s="396"/>
-      <c r="J7" s="396"/>
-      <c r="K7" s="396"/>
-      <c r="L7" s="396"/>
-      <c r="M7" s="396"/>
-      <c r="N7" s="396"/>
-      <c r="O7" s="396"/>
-      <c r="P7" s="396"/>
-      <c r="Q7" s="396"/>
-      <c r="R7" s="396"/>
-      <c r="S7" s="396"/>
-      <c r="T7" s="396"/>
-      <c r="U7" s="396"/>
-      <c r="V7" s="406"/>
-      <c r="W7" s="432"/>
-      <c r="X7" s="396"/>
-      <c r="Y7" s="396"/>
-      <c r="Z7" s="396"/>
-      <c r="AA7" s="396"/>
-      <c r="AB7" s="396"/>
-      <c r="AC7" s="396"/>
-      <c r="AD7" s="396"/>
-      <c r="AE7" s="396"/>
-      <c r="AF7" s="396"/>
-      <c r="AG7" s="396"/>
-      <c r="AH7" s="396"/>
-      <c r="AI7" s="396"/>
-      <c r="AJ7" s="396"/>
-      <c r="AK7" s="405"/>
-      <c r="AL7" s="396"/>
-      <c r="AM7" s="396"/>
-      <c r="AN7" s="396"/>
-      <c r="AO7" s="396"/>
-      <c r="AP7" s="396"/>
-      <c r="AQ7" s="396"/>
-      <c r="AR7" s="396"/>
-      <c r="AS7" s="396"/>
-      <c r="AT7" s="396"/>
-      <c r="AU7" s="396"/>
-      <c r="AV7" s="396"/>
-      <c r="AW7" s="396"/>
-      <c r="AX7" s="396"/>
+      <c r="A7" s="394"/>
+      <c r="B7" s="394"/>
+      <c r="C7" s="394"/>
+      <c r="D7" s="394"/>
+      <c r="E7" s="394"/>
+      <c r="F7" s="394"/>
+      <c r="G7" s="394"/>
+      <c r="H7" s="394"/>
+      <c r="I7" s="394"/>
+      <c r="J7" s="394"/>
+      <c r="K7" s="394"/>
+      <c r="L7" s="394"/>
+      <c r="M7" s="394"/>
+      <c r="N7" s="394"/>
+      <c r="O7" s="394"/>
+      <c r="P7" s="394"/>
+      <c r="Q7" s="394"/>
+      <c r="R7" s="394"/>
+      <c r="S7" s="394"/>
+      <c r="T7" s="394"/>
+      <c r="U7" s="394"/>
+      <c r="V7" s="404"/>
+      <c r="W7" s="430"/>
+      <c r="X7" s="394"/>
+      <c r="Y7" s="394"/>
+      <c r="Z7" s="394"/>
+      <c r="AA7" s="394"/>
+      <c r="AB7" s="394"/>
+      <c r="AC7" s="394"/>
+      <c r="AD7" s="394"/>
+      <c r="AE7" s="394"/>
+      <c r="AF7" s="394"/>
+      <c r="AG7" s="394"/>
+      <c r="AH7" s="394"/>
+      <c r="AI7" s="394"/>
+      <c r="AJ7" s="394"/>
+      <c r="AK7" s="403"/>
+      <c r="AL7" s="394"/>
+      <c r="AM7" s="394"/>
+      <c r="AN7" s="394"/>
+      <c r="AO7" s="394"/>
+      <c r="AP7" s="394"/>
+      <c r="AQ7" s="394"/>
+      <c r="AR7" s="394"/>
+      <c r="AS7" s="394"/>
+      <c r="AT7" s="394"/>
+      <c r="AU7" s="394"/>
+      <c r="AV7" s="394"/>
+      <c r="AW7" s="394"/>
+      <c r="AX7" s="394"/>
       <c r="AY7" s="29" t="s">
         <v>67</v>
       </c>
@@ -19168,122 +19160,122 @@
       <c r="BA7" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="410" t="s">
+      <c r="BB7" s="408" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="402" t="s">
+      <c r="BC7" s="400" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="402" t="s">
+      <c r="BD7" s="400" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="402" t="s">
+      <c r="BE7" s="400" t="s">
         <v>145</v>
       </c>
-      <c r="BF7" s="402" t="s">
+      <c r="BF7" s="400" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="402" t="s">
+      <c r="BG7" s="400" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="402" t="s">
+      <c r="BH7" s="400" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="402" t="s">
+      <c r="BI7" s="400" t="s">
         <v>79</v>
       </c>
-      <c r="BJ7" s="403" t="s">
+      <c r="BJ7" s="401" t="s">
         <v>80</v>
       </c>
-      <c r="BK7" s="402" t="s">
+      <c r="BK7" s="400" t="s">
         <v>81</v>
       </c>
-      <c r="BL7" s="410" t="s">
+      <c r="BL7" s="408" t="s">
         <v>82</v>
       </c>
-      <c r="BM7" s="402" t="s">
+      <c r="BM7" s="400" t="s">
         <v>83</v>
       </c>
-      <c r="BN7" s="410" t="s">
+      <c r="BN7" s="408" t="s">
         <v>84</v>
       </c>
-      <c r="BO7" s="410" t="s">
+      <c r="BO7" s="408" t="s">
         <v>146</v>
       </c>
-      <c r="BP7" s="410" t="s">
+      <c r="BP7" s="408" t="s">
         <v>85</v>
       </c>
-      <c r="BQ7" s="396"/>
-      <c r="BR7" s="396"/>
-      <c r="BS7" s="396"/>
-      <c r="BT7" s="396"/>
-      <c r="BU7" s="405"/>
-      <c r="BW7" s="408"/>
-      <c r="BX7" s="421"/>
-      <c r="BY7" s="422"/>
-      <c r="BZ7" s="422"/>
-      <c r="CA7" s="409"/>
-      <c r="CB7" s="396"/>
-      <c r="CC7" s="396"/>
-      <c r="CD7" s="396"/>
+      <c r="BQ7" s="394"/>
+      <c r="BR7" s="394"/>
+      <c r="BS7" s="394"/>
+      <c r="BT7" s="394"/>
+      <c r="BU7" s="403"/>
+      <c r="BW7" s="406"/>
+      <c r="BX7" s="419"/>
+      <c r="BY7" s="420"/>
+      <c r="BZ7" s="420"/>
+      <c r="CA7" s="407"/>
+      <c r="CB7" s="394"/>
+      <c r="CC7" s="394"/>
+      <c r="CD7" s="394"/>
       <c r="CH7" s="46"/>
       <c r="CI7" s="47"/>
     </row>
     <row r="8" spans="1:87" s="45" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A8" s="399"/>
-      <c r="B8" s="399"/>
-      <c r="C8" s="399"/>
-      <c r="D8" s="399"/>
-      <c r="E8" s="399"/>
-      <c r="F8" s="399"/>
-      <c r="G8" s="399"/>
-      <c r="H8" s="399"/>
-      <c r="I8" s="399"/>
-      <c r="J8" s="399"/>
-      <c r="K8" s="399"/>
-      <c r="L8" s="399"/>
-      <c r="M8" s="399"/>
-      <c r="N8" s="399"/>
-      <c r="O8" s="399"/>
-      <c r="P8" s="399"/>
-      <c r="Q8" s="399"/>
-      <c r="R8" s="399"/>
-      <c r="S8" s="399"/>
-      <c r="T8" s="399"/>
-      <c r="U8" s="399"/>
+      <c r="A8" s="397"/>
+      <c r="B8" s="397"/>
+      <c r="C8" s="397"/>
+      <c r="D8" s="397"/>
+      <c r="E8" s="397"/>
+      <c r="F8" s="397"/>
+      <c r="G8" s="397"/>
+      <c r="H8" s="397"/>
+      <c r="I8" s="397"/>
+      <c r="J8" s="397"/>
+      <c r="K8" s="397"/>
+      <c r="L8" s="397"/>
+      <c r="M8" s="397"/>
+      <c r="N8" s="397"/>
+      <c r="O8" s="397"/>
+      <c r="P8" s="397"/>
+      <c r="Q8" s="397"/>
+      <c r="R8" s="397"/>
+      <c r="S8" s="397"/>
+      <c r="T8" s="397"/>
+      <c r="U8" s="397"/>
       <c r="V8" s="49" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="399"/>
-      <c r="Y8" s="399"/>
-      <c r="Z8" s="399"/>
-      <c r="AA8" s="399"/>
-      <c r="AB8" s="399"/>
-      <c r="AC8" s="399"/>
-      <c r="AD8" s="399"/>
-      <c r="AE8" s="399"/>
-      <c r="AF8" s="399"/>
-      <c r="AG8" s="399"/>
-      <c r="AH8" s="399"/>
-      <c r="AI8" s="399"/>
-      <c r="AJ8" s="399"/>
-      <c r="AK8" s="406"/>
-      <c r="AL8" s="399"/>
-      <c r="AM8" s="399"/>
-      <c r="AN8" s="399"/>
-      <c r="AO8" s="399"/>
-      <c r="AP8" s="399"/>
-      <c r="AQ8" s="399"/>
-      <c r="AR8" s="399"/>
-      <c r="AS8" s="399"/>
-      <c r="AT8" s="399"/>
-      <c r="AU8" s="399"/>
-      <c r="AV8" s="399"/>
-      <c r="AW8" s="399"/>
-      <c r="AX8" s="399"/>
+      <c r="X8" s="397"/>
+      <c r="Y8" s="397"/>
+      <c r="Z8" s="397"/>
+      <c r="AA8" s="397"/>
+      <c r="AB8" s="397"/>
+      <c r="AC8" s="397"/>
+      <c r="AD8" s="397"/>
+      <c r="AE8" s="397"/>
+      <c r="AF8" s="397"/>
+      <c r="AG8" s="397"/>
+      <c r="AH8" s="397"/>
+      <c r="AI8" s="397"/>
+      <c r="AJ8" s="397"/>
+      <c r="AK8" s="404"/>
+      <c r="AL8" s="397"/>
+      <c r="AM8" s="397"/>
+      <c r="AN8" s="397"/>
+      <c r="AO8" s="397"/>
+      <c r="AP8" s="397"/>
+      <c r="AQ8" s="397"/>
+      <c r="AR8" s="397"/>
+      <c r="AS8" s="397"/>
+      <c r="AT8" s="397"/>
+      <c r="AU8" s="397"/>
+      <c r="AV8" s="397"/>
+      <c r="AW8" s="397"/>
+      <c r="AX8" s="397"/>
       <c r="AY8" s="30" t="s">
         <v>88</v>
       </c>
@@ -19293,27 +19285,27 @@
       <c r="BA8" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="399"/>
-      <c r="BC8" s="399"/>
-      <c r="BD8" s="399"/>
-      <c r="BE8" s="399"/>
-      <c r="BF8" s="399"/>
-      <c r="BG8" s="399"/>
-      <c r="BH8" s="399"/>
-      <c r="BI8" s="399"/>
-      <c r="BJ8" s="399"/>
-      <c r="BK8" s="399"/>
-      <c r="BL8" s="399"/>
-      <c r="BM8" s="399"/>
-      <c r="BN8" s="399"/>
-      <c r="BO8" s="399"/>
-      <c r="BP8" s="399"/>
-      <c r="BQ8" s="399"/>
-      <c r="BR8" s="399"/>
-      <c r="BS8" s="399"/>
-      <c r="BT8" s="399"/>
-      <c r="BU8" s="406"/>
-      <c r="BW8" s="409"/>
+      <c r="BB8" s="397"/>
+      <c r="BC8" s="397"/>
+      <c r="BD8" s="397"/>
+      <c r="BE8" s="397"/>
+      <c r="BF8" s="397"/>
+      <c r="BG8" s="397"/>
+      <c r="BH8" s="397"/>
+      <c r="BI8" s="397"/>
+      <c r="BJ8" s="397"/>
+      <c r="BK8" s="397"/>
+      <c r="BL8" s="397"/>
+      <c r="BM8" s="397"/>
+      <c r="BN8" s="397"/>
+      <c r="BO8" s="397"/>
+      <c r="BP8" s="397"/>
+      <c r="BQ8" s="397"/>
+      <c r="BR8" s="397"/>
+      <c r="BS8" s="397"/>
+      <c r="BT8" s="397"/>
+      <c r="BU8" s="404"/>
+      <c r="BW8" s="407"/>
       <c r="BX8" s="23" t="s">
         <v>91</v>
       </c>
@@ -19326,9 +19318,9 @@
       <c r="CA8" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="397"/>
-      <c r="CC8" s="397"/>
-      <c r="CD8" s="397"/>
+      <c r="CB8" s="395"/>
+      <c r="CC8" s="395"/>
+      <c r="CD8" s="395"/>
       <c r="CF8" s="50"/>
       <c r="CH8" s="46"/>
       <c r="CI8" s="47"/>

</xml_diff>